<commit_message>
20th dec data update
</commit_message>
<xml_diff>
--- a/Food Log Main.xlsx
+++ b/Food Log Main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91998\VS\Food Log Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F1EEBD-A345-4042-BEEC-EF52AA19AD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109D1D15-3DDC-403C-8A36-C8D828244616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Format 12 oct" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1595" uniqueCount="845">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1693" uniqueCount="897">
   <si>
     <t>date</t>
   </si>
@@ -2593,6 +2593,162 @@
   </si>
   <si>
     <t>WK20241212-p750</t>
+  </si>
+  <si>
+    <t>FD20241216-0800-q5r6</t>
+  </si>
+  <si>
+    <t>FD20241216-0900-s7t8</t>
+  </si>
+  <si>
+    <t>FD20241216-1200-u9v0</t>
+  </si>
+  <si>
+    <t>FD20241216-1230-w1x2</t>
+  </si>
+  <si>
+    <t>FD20241216-1500-y3z4</t>
+  </si>
+  <si>
+    <t>FD20241216-1830-a5b6</t>
+  </si>
+  <si>
+    <t>FD20241216-1900-c7d8</t>
+  </si>
+  <si>
+    <t>½ Starter 1</t>
+  </si>
+  <si>
+    <t>FD20241216-1930-e9f0</t>
+  </si>
+  <si>
+    <t>FD20241216-2100-g1h2</t>
+  </si>
+  <si>
+    <t>FD20241217-0730-i3j4</t>
+  </si>
+  <si>
+    <t>FD20241217-1000-k5l6</t>
+  </si>
+  <si>
+    <t>FD20241217-1300-m7n8</t>
+  </si>
+  <si>
+    <t>FD20241217-1300-o9p0</t>
+  </si>
+  <si>
+    <t>FD20241217-1400-q1r2</t>
+  </si>
+  <si>
+    <t>FD20241217-2130-s3t4</t>
+  </si>
+  <si>
+    <t>FD20241217-2200-u5v6</t>
+  </si>
+  <si>
+    <t>FD20241217-2230-w7x8</t>
+  </si>
+  <si>
+    <t>FD20241217-2330-y9z0</t>
+  </si>
+  <si>
+    <t>2 rotis with butter and 10g jaggery</t>
+  </si>
+  <si>
+    <t>FD20241218-0830-a1b2</t>
+  </si>
+  <si>
+    <t>FD20241218-0900-c3d4</t>
+  </si>
+  <si>
+    <t>FD20241218-1300-e5f6</t>
+  </si>
+  <si>
+    <t>FD20241218-1330-g7h8</t>
+  </si>
+  <si>
+    <t>FD20241218-1900-i9j0</t>
+  </si>
+  <si>
+    <t>FD20241218-1930-k1l2</t>
+  </si>
+  <si>
+    <t>FD20241218-2000-m3n4</t>
+  </si>
+  <si>
+    <t>FD20241218-2030-o5p6</t>
+  </si>
+  <si>
+    <t>FD20241219-0800-q7r8</t>
+  </si>
+  <si>
+    <t>FD20241219-0900-y5z6</t>
+  </si>
+  <si>
+    <t>FD20241219-1300-s9t0</t>
+  </si>
+  <si>
+    <t>FD20241219-1330-u1v2</t>
+  </si>
+  <si>
+    <t>FD20241219-1400-w3x4</t>
+  </si>
+  <si>
+    <t>FD20241219-1430-a7b8</t>
+  </si>
+  <si>
+    <t>FD20241219-1600-c9d0</t>
+  </si>
+  <si>
+    <t>FD20241219-1830-e1f2</t>
+  </si>
+  <si>
+    <t>FD20241219-1900-g3h4</t>
+  </si>
+  <si>
+    <t>FD20241219-1930-i5j6</t>
+  </si>
+  <si>
+    <t>FD20241219-2200-k7l8</t>
+  </si>
+  <si>
+    <t>FD20241220-0800-m7n8</t>
+  </si>
+  <si>
+    <t>FD20241220-1400-o9p0</t>
+  </si>
+  <si>
+    <t>3 servings of Brownie</t>
+  </si>
+  <si>
+    <t>FD20241220-1800-q1r2</t>
+  </si>
+  <si>
+    <t>FD20241220-1830-s3t4</t>
+  </si>
+  <si>
+    <t>FD20241220-1900-u5v6</t>
+  </si>
+  <si>
+    <t>2 rotis with butter and jaggery powder</t>
+  </si>
+  <si>
+    <t>1000133317.jpg</t>
+  </si>
+  <si>
+    <t>1000133851.jpg</t>
+  </si>
+  <si>
+    <t>WK20241216-p750</t>
+  </si>
+  <si>
+    <t>WK20241217-p1300</t>
+  </si>
+  <si>
+    <t>WK20241219-p925</t>
+  </si>
+  <si>
+    <t>WK20241220-wm</t>
   </si>
 </sst>
 </file>
@@ -3037,7 +3193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K546"/>
+  <dimension ref="A1:K588"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -20962,6 +21118,1350 @@
         <v>5.4</v>
       </c>
     </row>
+    <row r="547" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A547" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B547" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C547" s="2" t="s">
+        <v>845</v>
+      </c>
+      <c r="D547" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E547" s="2">
+        <v>77</v>
+      </c>
+      <c r="F547" s="2">
+        <v>2</v>
+      </c>
+      <c r="G547" s="2">
+        <v>11</v>
+      </c>
+      <c r="H547" s="2">
+        <v>2</v>
+      </c>
+      <c r="I547" s="2">
+        <v>7</v>
+      </c>
+      <c r="J547" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A548" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B548" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="C548" s="2" t="s">
+        <v>846</v>
+      </c>
+      <c r="D548" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E548" s="2">
+        <v>256</v>
+      </c>
+      <c r="F548" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="G548" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="H548" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="I548" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="J548" s="2">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="549" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A549" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B549" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="C549" s="2" t="s">
+        <v>847</v>
+      </c>
+      <c r="D549" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E549" s="2">
+        <v>290</v>
+      </c>
+      <c r="F549" s="2">
+        <v>11</v>
+      </c>
+      <c r="G549" s="2">
+        <v>18</v>
+      </c>
+      <c r="H549" s="2">
+        <v>18</v>
+      </c>
+      <c r="I549" s="2">
+        <v>0</v>
+      </c>
+      <c r="J549" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="550" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A550" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B550" s="17">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="C550" s="2" t="s">
+        <v>848</v>
+      </c>
+      <c r="D550" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E550" s="2">
+        <v>155</v>
+      </c>
+      <c r="F550" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G550" s="2">
+        <v>15</v>
+      </c>
+      <c r="H550" s="2">
+        <v>2</v>
+      </c>
+      <c r="I550" s="2">
+        <v>7</v>
+      </c>
+      <c r="J550" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="551" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A551" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B551" s="17">
+        <v>0.625</v>
+      </c>
+      <c r="C551" s="2" t="s">
+        <v>849</v>
+      </c>
+      <c r="D551" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E551" s="2">
+        <v>77</v>
+      </c>
+      <c r="F551" s="2">
+        <v>2</v>
+      </c>
+      <c r="G551" s="2">
+        <v>11</v>
+      </c>
+      <c r="H551" s="2">
+        <v>2</v>
+      </c>
+      <c r="I551" s="2">
+        <v>7</v>
+      </c>
+      <c r="J551" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="552" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A552" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B552" s="17">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C552" s="2" t="s">
+        <v>850</v>
+      </c>
+      <c r="D552" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E552" s="2">
+        <v>670</v>
+      </c>
+      <c r="F552" s="2">
+        <v>42</v>
+      </c>
+      <c r="G552" s="2">
+        <v>66</v>
+      </c>
+      <c r="H552" s="2">
+        <v>26</v>
+      </c>
+      <c r="I552" s="2">
+        <v>5</v>
+      </c>
+      <c r="J552" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="553" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A553" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B553" s="17">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C553" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="D553" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="E553" s="2">
+        <v>145</v>
+      </c>
+      <c r="F553" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="G553" s="2">
+        <v>9</v>
+      </c>
+      <c r="H553" s="2">
+        <v>9</v>
+      </c>
+      <c r="I553" s="2">
+        <v>0</v>
+      </c>
+      <c r="J553" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="554" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A554" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B554" s="17">
+        <v>0.8125</v>
+      </c>
+      <c r="C554" s="2" t="s">
+        <v>853</v>
+      </c>
+      <c r="D554" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E554" s="2">
+        <v>175</v>
+      </c>
+      <c r="F554" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G554" s="2">
+        <v>20</v>
+      </c>
+      <c r="H554" s="2">
+        <v>2</v>
+      </c>
+      <c r="I554" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="J554" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="555" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A555" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B555" s="17">
+        <v>0.875</v>
+      </c>
+      <c r="C555" s="2" t="s">
+        <v>854</v>
+      </c>
+      <c r="D555" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E555" s="2">
+        <v>128</v>
+      </c>
+      <c r="F555" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="G555" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="H555" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="I555" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J555" s="2">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="556" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A556" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B556" s="17">
+        <v>0.3125</v>
+      </c>
+      <c r="C556" s="2" t="s">
+        <v>855</v>
+      </c>
+      <c r="D556" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E556" s="2">
+        <v>77</v>
+      </c>
+      <c r="F556" s="2">
+        <v>2</v>
+      </c>
+      <c r="G556" s="2">
+        <v>11</v>
+      </c>
+      <c r="H556" s="2">
+        <v>2</v>
+      </c>
+      <c r="I556" s="2">
+        <v>7</v>
+      </c>
+      <c r="J556" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="557" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A557" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B557" s="17">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C557" s="2" t="s">
+        <v>856</v>
+      </c>
+      <c r="D557" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E557" s="2">
+        <v>128</v>
+      </c>
+      <c r="F557" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="G557" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="H557" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="I557" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J557" s="2">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="558" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A558" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B558" s="17">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C558" s="2" t="s">
+        <v>857</v>
+      </c>
+      <c r="D558" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E558" s="2">
+        <v>290</v>
+      </c>
+      <c r="F558" s="2">
+        <v>11</v>
+      </c>
+      <c r="G558" s="2">
+        <v>18</v>
+      </c>
+      <c r="H558" s="2">
+        <v>18</v>
+      </c>
+      <c r="I558" s="2">
+        <v>0</v>
+      </c>
+      <c r="J558" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="559" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A559" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B559" s="17">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C559" s="2" t="s">
+        <v>858</v>
+      </c>
+      <c r="D559" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E559" s="2">
+        <v>380</v>
+      </c>
+      <c r="F559" s="2">
+        <v>25</v>
+      </c>
+      <c r="G559" s="2">
+        <v>46</v>
+      </c>
+      <c r="H559" s="2">
+        <v>10</v>
+      </c>
+      <c r="I559" s="2">
+        <v>2</v>
+      </c>
+      <c r="J559" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="560" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A560" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B560" s="17">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C560" s="2" t="s">
+        <v>859</v>
+      </c>
+      <c r="D560" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E560" s="2">
+        <v>175</v>
+      </c>
+      <c r="F560" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G560" s="2">
+        <v>20</v>
+      </c>
+      <c r="H560" s="2">
+        <v>2</v>
+      </c>
+      <c r="I560" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="J560" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="561" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A561" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B561" s="17">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="C561" s="2" t="s">
+        <v>860</v>
+      </c>
+      <c r="D561" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E561" s="2">
+        <v>670</v>
+      </c>
+      <c r="F561" s="2">
+        <v>42</v>
+      </c>
+      <c r="G561" s="2">
+        <v>66</v>
+      </c>
+      <c r="H561" s="2">
+        <v>26</v>
+      </c>
+      <c r="I561" s="2">
+        <v>5</v>
+      </c>
+      <c r="J561" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="562" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A562" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B562" s="17">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C562" s="2" t="s">
+        <v>861</v>
+      </c>
+      <c r="D562" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E562" s="2">
+        <v>175</v>
+      </c>
+      <c r="F562" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G562" s="2">
+        <v>20</v>
+      </c>
+      <c r="H562" s="2">
+        <v>2</v>
+      </c>
+      <c r="I562" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="J562" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="563" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A563" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B563" s="17">
+        <v>0.9375</v>
+      </c>
+      <c r="C563" s="2" t="s">
+        <v>862</v>
+      </c>
+      <c r="D563" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E563" s="2">
+        <v>256</v>
+      </c>
+      <c r="F563" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="G563" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="H563" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="I563" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="J563" s="2">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="564" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A564" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B564" s="17">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="C564" s="2" t="s">
+        <v>863</v>
+      </c>
+      <c r="D564" s="2" t="s">
+        <v>864</v>
+      </c>
+      <c r="E564" s="2">
+        <v>370</v>
+      </c>
+      <c r="F564" s="2">
+        <v>6</v>
+      </c>
+      <c r="G564" s="2">
+        <v>55</v>
+      </c>
+      <c r="H564" s="2">
+        <v>13</v>
+      </c>
+      <c r="I564" s="2">
+        <v>21</v>
+      </c>
+      <c r="J564" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="565" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A565" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B565" s="17">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="C565" s="2" t="s">
+        <v>865</v>
+      </c>
+      <c r="D565" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E565" s="2">
+        <v>77</v>
+      </c>
+      <c r="F565" s="2">
+        <v>2</v>
+      </c>
+      <c r="G565" s="2">
+        <v>11</v>
+      </c>
+      <c r="H565" s="2">
+        <v>2</v>
+      </c>
+      <c r="I565" s="2">
+        <v>7</v>
+      </c>
+      <c r="J565" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="566" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A566" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B566" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="C566" s="2" t="s">
+        <v>866</v>
+      </c>
+      <c r="D566" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E566" s="2">
+        <v>256</v>
+      </c>
+      <c r="F566" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="G566" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="H566" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="I566" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="J566" s="2">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="567" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A567" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B567" s="17">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C567" s="2" t="s">
+        <v>867</v>
+      </c>
+      <c r="D567" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E567" s="2">
+        <v>290</v>
+      </c>
+      <c r="F567" s="2">
+        <v>11</v>
+      </c>
+      <c r="G567" s="2">
+        <v>18</v>
+      </c>
+      <c r="H567" s="2">
+        <v>18</v>
+      </c>
+      <c r="I567" s="2">
+        <v>0</v>
+      </c>
+      <c r="J567" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="568" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A568" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B568" s="17">
+        <v>0.5625</v>
+      </c>
+      <c r="C568" s="2" t="s">
+        <v>868</v>
+      </c>
+      <c r="D568" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E568" s="2">
+        <v>155</v>
+      </c>
+      <c r="F568" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G568" s="2">
+        <v>15</v>
+      </c>
+      <c r="H568" s="2">
+        <v>2</v>
+      </c>
+      <c r="I568" s="2">
+        <v>7</v>
+      </c>
+      <c r="J568" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="569" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A569" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B569" s="17">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C569" s="2" t="s">
+        <v>869</v>
+      </c>
+      <c r="D569" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E569" s="2">
+        <v>670</v>
+      </c>
+      <c r="F569" s="2">
+        <v>42</v>
+      </c>
+      <c r="G569" s="2">
+        <v>66</v>
+      </c>
+      <c r="H569" s="2">
+        <v>26</v>
+      </c>
+      <c r="I569" s="2">
+        <v>5</v>
+      </c>
+      <c r="J569" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="570" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A570" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B570" s="17">
+        <v>0.8125</v>
+      </c>
+      <c r="C570" s="2" t="s">
+        <v>870</v>
+      </c>
+      <c r="D570" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="E570" s="2">
+        <v>145</v>
+      </c>
+      <c r="F570" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="G570" s="2">
+        <v>9</v>
+      </c>
+      <c r="H570" s="2">
+        <v>9</v>
+      </c>
+      <c r="I570" s="2">
+        <v>0</v>
+      </c>
+      <c r="J570" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="571" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A571" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B571" s="17">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C571" s="2" t="s">
+        <v>871</v>
+      </c>
+      <c r="D571" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E571" s="2">
+        <v>175</v>
+      </c>
+      <c r="F571" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G571" s="2">
+        <v>20</v>
+      </c>
+      <c r="H571" s="2">
+        <v>2</v>
+      </c>
+      <c r="I571" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="J571" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="572" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A572" s="16">
+        <v>46009</v>
+      </c>
+      <c r="B572" s="17">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="C572" s="2" t="s">
+        <v>872</v>
+      </c>
+      <c r="D572" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E572" s="2">
+        <v>256</v>
+      </c>
+      <c r="F572" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="G572" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="H572" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="I572" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="J572" s="2">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="573" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A573" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B573" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C573" s="2" t="s">
+        <v>873</v>
+      </c>
+      <c r="D573" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E573" s="2">
+        <v>77</v>
+      </c>
+      <c r="F573" s="2">
+        <v>2</v>
+      </c>
+      <c r="G573" s="2">
+        <v>11</v>
+      </c>
+      <c r="H573" s="2">
+        <v>2</v>
+      </c>
+      <c r="I573" s="2">
+        <v>7</v>
+      </c>
+      <c r="J573" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="574" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A574" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B574" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="C574" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="D574" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="E574" s="2">
+        <v>105</v>
+      </c>
+      <c r="F574" s="2">
+        <v>2.6</v>
+      </c>
+      <c r="G574" s="2">
+        <v>21</v>
+      </c>
+      <c r="H574" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I574" s="2">
+        <v>14</v>
+      </c>
+      <c r="J574" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="575" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A575" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B575" s="17">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C575" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="D575" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E575" s="2">
+        <v>290</v>
+      </c>
+      <c r="F575" s="2">
+        <v>11</v>
+      </c>
+      <c r="G575" s="2">
+        <v>18</v>
+      </c>
+      <c r="H575" s="2">
+        <v>18</v>
+      </c>
+      <c r="I575" s="2">
+        <v>0</v>
+      </c>
+      <c r="J575" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="576" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A576" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B576" s="17">
+        <v>0.5625</v>
+      </c>
+      <c r="C576" s="2" t="s">
+        <v>876</v>
+      </c>
+      <c r="D576" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E576" s="2">
+        <v>380</v>
+      </c>
+      <c r="F576" s="2">
+        <v>25</v>
+      </c>
+      <c r="G576" s="2">
+        <v>46</v>
+      </c>
+      <c r="H576" s="2">
+        <v>10</v>
+      </c>
+      <c r="I576" s="2">
+        <v>2</v>
+      </c>
+      <c r="J576" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="577" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A577" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B577" s="17">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C577" s="2" t="s">
+        <v>877</v>
+      </c>
+      <c r="D577" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E577" s="2">
+        <v>155</v>
+      </c>
+      <c r="F577" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G577" s="2">
+        <v>15</v>
+      </c>
+      <c r="H577" s="2">
+        <v>2</v>
+      </c>
+      <c r="I577" s="2">
+        <v>7</v>
+      </c>
+      <c r="J577" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="578" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A578" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B578" s="17">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C578" s="2" t="s">
+        <v>878</v>
+      </c>
+      <c r="D578" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="E578" s="2">
+        <v>105</v>
+      </c>
+      <c r="F578" s="2">
+        <v>2.6</v>
+      </c>
+      <c r="G578" s="2">
+        <v>21</v>
+      </c>
+      <c r="H578" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="I578" s="2">
+        <v>14</v>
+      </c>
+      <c r="J578" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="579" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A579" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B579" s="17">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C579" s="2" t="s">
+        <v>879</v>
+      </c>
+      <c r="D579" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E579" s="2">
+        <v>77</v>
+      </c>
+      <c r="F579" s="2">
+        <v>2</v>
+      </c>
+      <c r="G579" s="2">
+        <v>11</v>
+      </c>
+      <c r="H579" s="2">
+        <v>2</v>
+      </c>
+      <c r="I579" s="2">
+        <v>7</v>
+      </c>
+      <c r="J579" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="580" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A580" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B580" s="17">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C580" s="2" t="s">
+        <v>880</v>
+      </c>
+      <c r="D580" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E580" s="2">
+        <v>670</v>
+      </c>
+      <c r="F580" s="2">
+        <v>42</v>
+      </c>
+      <c r="G580" s="2">
+        <v>66</v>
+      </c>
+      <c r="H580" s="2">
+        <v>26</v>
+      </c>
+      <c r="I580" s="2">
+        <v>5</v>
+      </c>
+      <c r="J580" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="581" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A581" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B581" s="17">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C581" s="2" t="s">
+        <v>881</v>
+      </c>
+      <c r="D581" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="E581" s="2">
+        <v>145</v>
+      </c>
+      <c r="F581" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="G581" s="2">
+        <v>9</v>
+      </c>
+      <c r="H581" s="2">
+        <v>9</v>
+      </c>
+      <c r="I581" s="2">
+        <v>0</v>
+      </c>
+      <c r="J581" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="582" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A582" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B582" s="17">
+        <v>0.8125</v>
+      </c>
+      <c r="C582" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="D582" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E582" s="2">
+        <v>128</v>
+      </c>
+      <c r="F582" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="G582" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="H582" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="I582" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J582" s="2">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="583" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A583" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B583" s="17">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C583" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="D583" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E583" s="2">
+        <v>158</v>
+      </c>
+      <c r="F583" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="G583" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="H583" s="2">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="I583" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="J583" s="2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="584" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A584" s="16">
+        <v>46011</v>
+      </c>
+      <c r="B584" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C584" s="2" t="s">
+        <v>884</v>
+      </c>
+      <c r="D584" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E584" s="2">
+        <v>77</v>
+      </c>
+      <c r="F584" s="2">
+        <v>2</v>
+      </c>
+      <c r="G584" s="2">
+        <v>11</v>
+      </c>
+      <c r="H584" s="2">
+        <v>2</v>
+      </c>
+      <c r="I584" s="2">
+        <v>7</v>
+      </c>
+      <c r="J584" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="585" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A585" s="16">
+        <v>46011</v>
+      </c>
+      <c r="B585" s="17">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C585" s="2" t="s">
+        <v>885</v>
+      </c>
+      <c r="D585" s="2" t="s">
+        <v>886</v>
+      </c>
+      <c r="E585" s="2">
+        <v>918</v>
+      </c>
+      <c r="F585" s="2">
+        <v>12.9</v>
+      </c>
+      <c r="G585" s="2">
+        <v>102.9</v>
+      </c>
+      <c r="H585" s="2">
+        <v>53.1</v>
+      </c>
+      <c r="I585" s="2">
+        <v>60</v>
+      </c>
+      <c r="J585" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="586" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A586" s="16">
+        <v>46011</v>
+      </c>
+      <c r="B586" s="17">
+        <v>0.75</v>
+      </c>
+      <c r="C586" s="2" t="s">
+        <v>887</v>
+      </c>
+      <c r="D586" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E586" s="2">
+        <v>670</v>
+      </c>
+      <c r="F586" s="2">
+        <v>42</v>
+      </c>
+      <c r="G586" s="2">
+        <v>66</v>
+      </c>
+      <c r="H586" s="2">
+        <v>26</v>
+      </c>
+      <c r="I586" s="2">
+        <v>5</v>
+      </c>
+      <c r="J586" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="587" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A587" s="16">
+        <v>46011</v>
+      </c>
+      <c r="B587" s="17">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C587" s="2" t="s">
+        <v>888</v>
+      </c>
+      <c r="D587" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E587" s="2">
+        <v>175</v>
+      </c>
+      <c r="F587" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G587" s="2">
+        <v>20</v>
+      </c>
+      <c r="H587" s="2">
+        <v>2</v>
+      </c>
+      <c r="I587" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="J587" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="588" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A588" s="16">
+        <v>46011</v>
+      </c>
+      <c r="B588" s="17">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C588" s="2" t="s">
+        <v>889</v>
+      </c>
+      <c r="D588" s="2" t="s">
+        <v>890</v>
+      </c>
+      <c r="E588" s="2">
+        <v>310</v>
+      </c>
+      <c r="F588" s="2">
+        <v>6</v>
+      </c>
+      <c r="G588" s="2">
+        <v>45</v>
+      </c>
+      <c r="H588" s="2">
+        <v>12</v>
+      </c>
+      <c r="I588" s="2">
+        <v>11</v>
+      </c>
+      <c r="J588" s="2">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="C277:C1048576 C1:C211 C217:C265">
@@ -20973,7 +22473,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F24E0C0-BC77-4AA4-801C-82B038A8B8E4}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -21484,6 +22984,46 @@
         <v>842</v>
       </c>
     </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B26" s="2">
+        <v>97.5</v>
+      </c>
+      <c r="C26" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="D26" s="2">
+        <v>30.5</v>
+      </c>
+      <c r="E26" s="2">
+        <v>49.1</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="16">
+        <v>46011</v>
+      </c>
+      <c r="B27" s="2">
+        <v>97.9</v>
+      </c>
+      <c r="C27" s="2">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="D27" s="2">
+        <v>28.9</v>
+      </c>
+      <c r="E27" s="2">
+        <v>50.6</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>892</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21492,7 +23032,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06D2F321-D2D4-48D2-B6F9-E306604CF730}">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -22020,7 +23560,9 @@
       <c r="D22" s="2">
         <v>30</v>
       </c>
-      <c r="E22" s="2"/>
+      <c r="E22" s="2">
+        <v>304</v>
+      </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2" t="s">
@@ -22040,7 +23582,9 @@
       <c r="D23" s="2">
         <v>51</v>
       </c>
-      <c r="E23" s="2"/>
+      <c r="E23" s="2">
+        <v>451</v>
+      </c>
       <c r="F23" s="2">
         <v>1075</v>
       </c>
@@ -22197,6 +23741,100 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2" t="s">
         <v>844</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="16">
+        <v>46007</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D30" s="2">
+        <v>40</v>
+      </c>
+      <c r="E30" s="2">
+        <v>370</v>
+      </c>
+      <c r="F30" s="2">
+        <v>750</v>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="16">
+        <v>46008</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D31" s="2">
+        <v>50</v>
+      </c>
+      <c r="E31" s="2">
+        <v>518</v>
+      </c>
+      <c r="F31" s="2">
+        <v>1300</v>
+      </c>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="16">
+        <v>46010</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" s="2">
+        <v>39</v>
+      </c>
+      <c r="E32" s="2">
+        <v>392</v>
+      </c>
+      <c r="F32" s="2">
+        <v>925</v>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="16">
+        <v>46011</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" s="2">
+        <v>50</v>
+      </c>
+      <c r="E33" s="2">
+        <v>374</v>
+      </c>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2" t="s">
+        <v>896</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
16th jan data update
</commit_message>
<xml_diff>
--- a/Food Log Main.xlsx
+++ b/Food Log Main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91998\VS\Food Log Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{731D474C-26BC-428D-9DE9-4D61943C3C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBABBD4-2BC1-46B1-9BDD-880EAFD590C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Format 12 oct" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Daily 23 to 11oct" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Main Format 12 oct'!#REF!</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Main Format 12 oct'!$A$806:$J$838</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Sheet1!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weight Tracker 23sep'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workouts 19oct'!$A$1:$H$1</definedName>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2353" uniqueCount="1185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2435" uniqueCount="1232">
   <si>
     <t>date</t>
   </si>
@@ -3615,6 +3615,147 @@
   </si>
   <si>
     <t>1000140850.jpg</t>
+  </si>
+  <si>
+    <t>FD20260114-0800-7f1a</t>
+  </si>
+  <si>
+    <t>FD20260114-0830-8g2b</t>
+  </si>
+  <si>
+    <t>FD20260114-1130-9h3c</t>
+  </si>
+  <si>
+    <t>FD20260114-1200-0i4d</t>
+  </si>
+  <si>
+    <t>FD20260114-1500-1j5e</t>
+  </si>
+  <si>
+    <t>2 boiled eggs</t>
+  </si>
+  <si>
+    <t>FD20260114-1530-2k6f</t>
+  </si>
+  <si>
+    <t>FD20260114-2000-3l7g</t>
+  </si>
+  <si>
+    <t>Banana (100g)</t>
+  </si>
+  <si>
+    <t>FD20260114-2030-4m8h</t>
+  </si>
+  <si>
+    <t>FD20260114-2130-5n9i</t>
+  </si>
+  <si>
+    <t>Chicken mushroom cream soup (330g) + breadsticks (19g)</t>
+  </si>
+  <si>
+    <t>FD20260114-2200-6o0j</t>
+  </si>
+  <si>
+    <t>FD20260114-2200-7p1k</t>
+  </si>
+  <si>
+    <t>FD20260115-0800-8q2l</t>
+  </si>
+  <si>
+    <t>FD20260115-0830-9r3m</t>
+  </si>
+  <si>
+    <t>FD20260115-1030-0s4n</t>
+  </si>
+  <si>
+    <t>Guava (150g)</t>
+  </si>
+  <si>
+    <t>FD20260115-1430-1t5o</t>
+  </si>
+  <si>
+    <t>FD20260115-1500-2u6p</t>
+  </si>
+  <si>
+    <t>FD20260115-1530-3v7q</t>
+  </si>
+  <si>
+    <t>FD20260115-1800-4w8r</t>
+  </si>
+  <si>
+    <t>FD20260115-2000-5x9s</t>
+  </si>
+  <si>
+    <t>Shake 2 (with 5g sugar)</t>
+  </si>
+  <si>
+    <t>FD20260115-2030-6y0t</t>
+  </si>
+  <si>
+    <t>FD20260116-0700-7z1u</t>
+  </si>
+  <si>
+    <t>FD20260116-0730-8a2v</t>
+  </si>
+  <si>
+    <t>FD20260116-0800-9b3w</t>
+  </si>
+  <si>
+    <t>FD20260116-0830-0c4x</t>
+  </si>
+  <si>
+    <t>1 roti with butter and jaggery</t>
+  </si>
+  <si>
+    <t>FD20260116-1100-1d5y</t>
+  </si>
+  <si>
+    <t>Milk coffee with 5g sugar</t>
+  </si>
+  <si>
+    <t>FD20260116-1130-2e6z</t>
+  </si>
+  <si>
+    <t>FD20260116-1200-3f7a</t>
+  </si>
+  <si>
+    <t>FD20260116-1400-4g8b</t>
+  </si>
+  <si>
+    <t>FD20260116-1700-5h9c</t>
+  </si>
+  <si>
+    <t>FD20260116-1730-6i0d</t>
+  </si>
+  <si>
+    <t>FD20260116-1800-7j1e</t>
+  </si>
+  <si>
+    <t>FD20260116-1830-8k2f</t>
+  </si>
+  <si>
+    <t>Mad Angles (30g)</t>
+  </si>
+  <si>
+    <t>FD20260116-1900-9l3g</t>
+  </si>
+  <si>
+    <t>1000139603.jpg</t>
+  </si>
+  <si>
+    <t>1000142235.jpg</t>
+  </si>
+  <si>
+    <t>WK20260114-wm</t>
+  </si>
+  <si>
+    <t>WK20260115-w</t>
+  </si>
+  <si>
+    <t>WK20260115-b</t>
+  </si>
+  <si>
+    <t>WK20260117-wm</t>
   </si>
 </sst>
 </file>
@@ -3684,7 +3825,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -3762,7 +3903,6 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4094,7 +4234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J805"/>
+  <dimension ref="A1:J838"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -27875,1987 +28015,3043 @@
       </c>
     </row>
     <row r="744" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A744" s="29">
+      <c r="A744" s="16">
         <v>46029</v>
       </c>
-      <c r="B744" s="30">
+      <c r="B744" s="17">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C744" t="s">
+      <c r="C744" s="2" t="s">
         <v>1103</v>
       </c>
-      <c r="D744" t="s">
+      <c r="D744" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E744">
+      <c r="E744" s="2">
         <v>77</v>
       </c>
-      <c r="F744">
-        <v>2</v>
-      </c>
-      <c r="G744">
+      <c r="F744" s="2">
+        <v>2</v>
+      </c>
+      <c r="G744" s="2">
         <v>11</v>
       </c>
-      <c r="H744">
-        <v>2</v>
-      </c>
-      <c r="I744">
+      <c r="H744" s="2">
+        <v>2</v>
+      </c>
+      <c r="I744" s="2">
         <v>7</v>
       </c>
-      <c r="J744">
+      <c r="J744" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="745" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A745" s="29">
+      <c r="A745" s="16">
         <v>46029</v>
       </c>
-      <c r="B745" s="30">
+      <c r="B745" s="17">
         <v>0.5</v>
       </c>
-      <c r="C745" t="s">
+      <c r="C745" s="2" t="s">
         <v>1104</v>
       </c>
-      <c r="D745" t="s">
+      <c r="D745" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E745">
+      <c r="E745" s="2">
         <v>290</v>
       </c>
-      <c r="F745">
+      <c r="F745" s="2">
         <v>11</v>
       </c>
-      <c r="G745">
+      <c r="G745" s="2">
         <v>18</v>
       </c>
-      <c r="H745">
+      <c r="H745" s="2">
         <v>18</v>
       </c>
-      <c r="I745">
+      <c r="I745" s="2">
         <v>0</v>
       </c>
-      <c r="J745">
+      <c r="J745" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="746" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A746" s="29">
+      <c r="A746" s="16">
         <v>46029</v>
       </c>
-      <c r="B746" s="30">
+      <c r="B746" s="17">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C746" t="s">
+      <c r="C746" s="2" t="s">
         <v>1105</v>
       </c>
-      <c r="D746" t="s">
+      <c r="D746" s="2" t="s">
         <v>917</v>
       </c>
-      <c r="E746">
+      <c r="E746" s="2">
         <v>502.5</v>
       </c>
-      <c r="F746">
+      <c r="F746" s="2">
         <v>31.5</v>
       </c>
-      <c r="G746">
+      <c r="G746" s="2">
         <v>49.5</v>
       </c>
-      <c r="H746">
+      <c r="H746" s="2">
         <v>19.5</v>
       </c>
-      <c r="I746">
+      <c r="I746" s="2">
         <v>3.75</v>
       </c>
-      <c r="J746">
+      <c r="J746" s="2">
         <v>3.75</v>
       </c>
     </row>
     <row r="747" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A747" s="29">
+      <c r="A747" s="16">
         <v>46029</v>
       </c>
-      <c r="B747" s="30">
+      <c r="B747" s="17">
         <v>0.5625</v>
       </c>
-      <c r="C747" t="s">
+      <c r="C747" s="2" t="s">
         <v>1106</v>
       </c>
-      <c r="D747" t="s">
+      <c r="D747" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E747">
+      <c r="E747" s="2">
         <v>155</v>
       </c>
-      <c r="F747">
+      <c r="F747" s="2">
         <v>15.5</v>
       </c>
-      <c r="G747">
+      <c r="G747" s="2">
         <v>15</v>
       </c>
-      <c r="H747">
-        <v>2</v>
-      </c>
-      <c r="I747">
+      <c r="H747" s="2">
+        <v>2</v>
+      </c>
+      <c r="I747" s="2">
         <v>7</v>
       </c>
-      <c r="J747">
+      <c r="J747" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="748" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A748" s="29">
+      <c r="A748" s="16">
         <v>46029</v>
       </c>
-      <c r="B748" s="30">
+      <c r="B748" s="17">
         <v>0.58333333333333337</v>
       </c>
-      <c r="C748" t="s">
+      <c r="C748" s="2" t="s">
         <v>1107</v>
       </c>
-      <c r="D748" t="s">
+      <c r="D748" s="2" t="s">
         <v>1056</v>
       </c>
-      <c r="E748">
+      <c r="E748" s="2">
         <v>165</v>
       </c>
-      <c r="F748">
+      <c r="F748" s="2">
         <v>5</v>
       </c>
-      <c r="G748">
+      <c r="G748" s="2">
         <v>9</v>
       </c>
-      <c r="H748">
+      <c r="H748" s="2">
         <v>13.5</v>
       </c>
-      <c r="I748">
+      <c r="I748" s="2">
         <v>1.5</v>
       </c>
-      <c r="J748">
+      <c r="J748" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="749" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A749" s="29">
+      <c r="A749" s="16">
         <v>46029</v>
       </c>
-      <c r="B749" s="30">
+      <c r="B749" s="17">
         <v>0.64583333333333337</v>
       </c>
-      <c r="C749" t="s">
+      <c r="C749" s="2" t="s">
         <v>1108</v>
       </c>
-      <c r="D749" t="s">
+      <c r="D749" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E749">
+      <c r="E749" s="2">
         <v>77</v>
       </c>
-      <c r="F749">
-        <v>2</v>
-      </c>
-      <c r="G749">
+      <c r="F749" s="2">
+        <v>2</v>
+      </c>
+      <c r="G749" s="2">
         <v>11</v>
       </c>
-      <c r="H749">
-        <v>2</v>
-      </c>
-      <c r="I749">
+      <c r="H749" s="2">
+        <v>2</v>
+      </c>
+      <c r="I749" s="2">
         <v>7</v>
       </c>
-      <c r="J749">
+      <c r="J749" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="750" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A750" s="29">
+      <c r="A750" s="16">
         <v>46029</v>
       </c>
-      <c r="B750" s="30">
+      <c r="B750" s="17">
         <v>0.8125</v>
       </c>
-      <c r="C750" t="s">
+      <c r="C750" s="2" t="s">
         <v>1109</v>
       </c>
-      <c r="D750" t="s">
+      <c r="D750" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E750">
+      <c r="E750" s="2">
         <v>380</v>
       </c>
-      <c r="F750">
+      <c r="F750" s="2">
         <v>25</v>
       </c>
-      <c r="G750">
+      <c r="G750" s="2">
         <v>46</v>
       </c>
-      <c r="H750">
+      <c r="H750" s="2">
         <v>10</v>
       </c>
-      <c r="I750">
-        <v>2</v>
-      </c>
-      <c r="J750">
+      <c r="I750" s="2">
+        <v>2</v>
+      </c>
+      <c r="J750" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="751" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A751" s="29">
+      <c r="A751" s="16">
         <v>46029</v>
       </c>
-      <c r="B751" s="30">
+      <c r="B751" s="17">
         <v>0.83333333333333337</v>
       </c>
-      <c r="C751" t="s">
+      <c r="C751" s="2" t="s">
         <v>1110</v>
       </c>
-      <c r="D751" t="s">
+      <c r="D751" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E751">
+      <c r="E751" s="2">
         <v>155</v>
       </c>
-      <c r="F751">
+      <c r="F751" s="2">
         <v>15.5</v>
       </c>
-      <c r="G751">
+      <c r="G751" s="2">
         <v>15</v>
       </c>
-      <c r="H751">
-        <v>2</v>
-      </c>
-      <c r="I751">
+      <c r="H751" s="2">
+        <v>2</v>
+      </c>
+      <c r="I751" s="2">
         <v>7</v>
       </c>
-      <c r="J751">
+      <c r="J751" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="752" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A752" s="29">
+      <c r="A752" s="16">
         <v>46030</v>
       </c>
-      <c r="B752" s="30">
+      <c r="B752" s="17">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C752" t="s">
+      <c r="C752" s="2" t="s">
         <v>1111</v>
       </c>
-      <c r="D752" t="s">
+      <c r="D752" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E752">
+      <c r="E752" s="2">
         <v>77</v>
       </c>
-      <c r="F752">
-        <v>2</v>
-      </c>
-      <c r="G752">
+      <c r="F752" s="2">
+        <v>2</v>
+      </c>
+      <c r="G752" s="2">
         <v>11</v>
       </c>
-      <c r="H752">
-        <v>2</v>
-      </c>
-      <c r="I752">
+      <c r="H752" s="2">
+        <v>2</v>
+      </c>
+      <c r="I752" s="2">
         <v>7</v>
       </c>
-      <c r="J752">
+      <c r="J752" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="753" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A753" s="29">
+      <c r="A753" s="16">
         <v>46030</v>
       </c>
-      <c r="B753" s="30">
+      <c r="B753" s="17">
         <v>0.35416666666666669</v>
       </c>
-      <c r="C753" t="s">
+      <c r="C753" s="2" t="s">
         <v>1112</v>
       </c>
-      <c r="D753" t="s">
+      <c r="D753" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E753">
+      <c r="E753" s="2">
         <v>128</v>
       </c>
-      <c r="F753">
+      <c r="F753" s="2">
         <v>6.6</v>
       </c>
-      <c r="G753">
+      <c r="G753" s="2">
         <v>9.6</v>
       </c>
-      <c r="H753">
+      <c r="H753" s="2">
         <v>5.3</v>
       </c>
-      <c r="I753">
+      <c r="I753" s="2">
         <v>5.3</v>
       </c>
-      <c r="J753">
+      <c r="J753" s="2">
         <v>2.7</v>
       </c>
     </row>
     <row r="754" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A754" s="29">
+      <c r="A754" s="16">
         <v>46030</v>
       </c>
-      <c r="B754" s="30">
+      <c r="B754" s="17">
         <v>0.375</v>
       </c>
-      <c r="C754" t="s">
+      <c r="C754" s="2" t="s">
         <v>1113</v>
       </c>
-      <c r="D754" t="s">
+      <c r="D754" s="2" t="s">
         <v>1114</v>
       </c>
-      <c r="E754">
+      <c r="E754" s="2">
         <v>82.5</v>
       </c>
-      <c r="F754">
+      <c r="F754" s="2">
         <v>2.5</v>
       </c>
-      <c r="G754">
+      <c r="G754" s="2">
         <v>4.5</v>
       </c>
-      <c r="H754">
+      <c r="H754" s="2">
         <v>6.75</v>
       </c>
-      <c r="I754">
+      <c r="I754" s="2">
         <v>0.75</v>
       </c>
-      <c r="J754">
+      <c r="J754" s="2">
         <v>0.5</v>
       </c>
     </row>
     <row r="755" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A755" s="29">
+      <c r="A755" s="16">
         <v>46030</v>
       </c>
-      <c r="B755" s="30">
+      <c r="B755" s="17">
         <v>0.52083333333333337</v>
       </c>
-      <c r="C755" t="s">
+      <c r="C755" s="2" t="s">
         <v>1115</v>
       </c>
-      <c r="D755" t="s">
+      <c r="D755" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E755">
+      <c r="E755" s="2">
         <v>290</v>
       </c>
-      <c r="F755">
+      <c r="F755" s="2">
         <v>11</v>
       </c>
-      <c r="G755">
+      <c r="G755" s="2">
         <v>18</v>
       </c>
-      <c r="H755">
+      <c r="H755" s="2">
         <v>18</v>
       </c>
-      <c r="I755">
+      <c r="I755" s="2">
         <v>0</v>
       </c>
-      <c r="J755">
+      <c r="J755" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="756" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A756" s="29">
+      <c r="A756" s="16">
         <v>46030</v>
       </c>
-      <c r="B756" s="30">
+      <c r="B756" s="17">
         <v>0.64583333333333337</v>
       </c>
-      <c r="C756" t="s">
+      <c r="C756" s="2" t="s">
         <v>1116</v>
       </c>
-      <c r="D756" t="s">
+      <c r="D756" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E756">
+      <c r="E756" s="2">
         <v>380</v>
       </c>
-      <c r="F756">
+      <c r="F756" s="2">
         <v>25</v>
       </c>
-      <c r="G756">
+      <c r="G756" s="2">
         <v>46</v>
       </c>
-      <c r="H756">
+      <c r="H756" s="2">
         <v>10</v>
       </c>
-      <c r="I756">
-        <v>2</v>
-      </c>
-      <c r="J756">
+      <c r="I756" s="2">
+        <v>2</v>
+      </c>
+      <c r="J756" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="757" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A757" s="29">
+      <c r="A757" s="16">
         <v>46030</v>
       </c>
-      <c r="B757" s="30">
+      <c r="B757" s="17">
         <v>0.66666666666666663</v>
       </c>
-      <c r="C757" t="s">
+      <c r="C757" s="2" t="s">
         <v>1117</v>
       </c>
-      <c r="D757" t="s">
+      <c r="D757" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E757">
+      <c r="E757" s="2">
         <v>155</v>
       </c>
-      <c r="F757">
+      <c r="F757" s="2">
         <v>15.5</v>
       </c>
-      <c r="G757">
+      <c r="G757" s="2">
         <v>15</v>
       </c>
-      <c r="H757">
-        <v>2</v>
-      </c>
-      <c r="I757">
+      <c r="H757" s="2">
+        <v>2</v>
+      </c>
+      <c r="I757" s="2">
         <v>7</v>
       </c>
-      <c r="J757">
+      <c r="J757" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="758" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A758" s="29">
+      <c r="A758" s="16">
         <v>46030</v>
       </c>
-      <c r="B758" s="30">
+      <c r="B758" s="17">
         <v>0.72916666666666663</v>
       </c>
-      <c r="C758" t="s">
+      <c r="C758" s="2" t="s">
         <v>1118</v>
       </c>
-      <c r="D758" t="s">
+      <c r="D758" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E758">
+      <c r="E758" s="2">
         <v>77</v>
       </c>
-      <c r="F758">
-        <v>2</v>
-      </c>
-      <c r="G758">
+      <c r="F758" s="2">
+        <v>2</v>
+      </c>
+      <c r="G758" s="2">
         <v>11</v>
       </c>
-      <c r="H758">
-        <v>2</v>
-      </c>
-      <c r="I758">
+      <c r="H758" s="2">
+        <v>2</v>
+      </c>
+      <c r="I758" s="2">
         <v>7</v>
       </c>
-      <c r="J758">
+      <c r="J758" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="759" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A759" s="29">
+      <c r="A759" s="16">
         <v>46030</v>
       </c>
-      <c r="B759" s="30">
+      <c r="B759" s="17">
         <v>0.75</v>
       </c>
-      <c r="C759" t="s">
+      <c r="C759" s="2" t="s">
         <v>1119</v>
       </c>
-      <c r="D759" t="s">
+      <c r="D759" s="2" t="s">
         <v>1114</v>
       </c>
-      <c r="E759">
+      <c r="E759" s="2">
         <v>82.5</v>
       </c>
-      <c r="F759">
+      <c r="F759" s="2">
         <v>2.5</v>
       </c>
-      <c r="G759">
+      <c r="G759" s="2">
         <v>4.5</v>
       </c>
-      <c r="H759">
+      <c r="H759" s="2">
         <v>6.75</v>
       </c>
-      <c r="I759">
+      <c r="I759" s="2">
         <v>0.75</v>
       </c>
-      <c r="J759">
+      <c r="J759" s="2">
         <v>0.5</v>
       </c>
     </row>
     <row r="760" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A760" s="29">
+      <c r="A760" s="16">
         <v>46030</v>
       </c>
-      <c r="B760" s="30">
+      <c r="B760" s="17">
         <v>0.77083333333333337</v>
       </c>
-      <c r="C760" t="s">
+      <c r="C760" s="2" t="s">
         <v>1120</v>
       </c>
-      <c r="D760" t="s">
+      <c r="D760" s="2" t="s">
         <v>808</v>
       </c>
-      <c r="E760">
+      <c r="E760" s="2">
         <v>145</v>
       </c>
-      <c r="F760">
+      <c r="F760" s="2">
         <v>5.5</v>
       </c>
-      <c r="G760">
+      <c r="G760" s="2">
         <v>9</v>
       </c>
-      <c r="H760">
+      <c r="H760" s="2">
         <v>9</v>
       </c>
-      <c r="I760">
+      <c r="I760" s="2">
         <v>0</v>
       </c>
-      <c r="J760">
+      <c r="J760" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="761" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A761" s="29">
+      <c r="A761" s="16">
         <v>46030</v>
       </c>
-      <c r="B761" s="30">
+      <c r="B761" s="17">
         <v>0.79166666666666663</v>
       </c>
-      <c r="C761" t="s">
+      <c r="C761" s="2" t="s">
         <v>1121</v>
       </c>
-      <c r="D761" t="s">
+      <c r="D761" s="2" t="s">
         <v>932</v>
       </c>
-      <c r="E761">
+      <c r="E761" s="2">
         <v>335</v>
       </c>
-      <c r="F761">
+      <c r="F761" s="2">
         <v>21</v>
       </c>
-      <c r="G761">
+      <c r="G761" s="2">
         <v>33</v>
       </c>
-      <c r="H761">
+      <c r="H761" s="2">
         <v>13</v>
       </c>
-      <c r="I761">
+      <c r="I761" s="2">
         <v>2.5</v>
       </c>
-      <c r="J761">
+      <c r="J761" s="2">
         <v>2.5</v>
       </c>
     </row>
     <row r="762" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A762" s="29">
+      <c r="A762" s="16">
         <v>46031</v>
       </c>
-      <c r="B762" s="30">
+      <c r="B762" s="17">
         <v>0.35416666666666669</v>
       </c>
-      <c r="C762" t="s">
+      <c r="C762" s="2" t="s">
         <v>1122</v>
       </c>
-      <c r="D762" t="s">
+      <c r="D762" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E762">
+      <c r="E762" s="2">
         <v>77</v>
       </c>
-      <c r="F762">
-        <v>2</v>
-      </c>
-      <c r="G762">
+      <c r="F762" s="2">
+        <v>2</v>
+      </c>
+      <c r="G762" s="2">
         <v>11</v>
       </c>
-      <c r="H762">
-        <v>2</v>
-      </c>
-      <c r="I762">
+      <c r="H762" s="2">
+        <v>2</v>
+      </c>
+      <c r="I762" s="2">
         <v>7</v>
       </c>
-      <c r="J762">
+      <c r="J762" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="763" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A763" s="29">
+      <c r="A763" s="16">
         <v>46031</v>
       </c>
-      <c r="B763" s="30">
+      <c r="B763" s="17">
         <v>0.39583333333333331</v>
       </c>
-      <c r="C763" t="s">
+      <c r="C763" s="2" t="s">
         <v>1123</v>
       </c>
-      <c r="D763" t="s">
+      <c r="D763" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E763">
+      <c r="E763" s="2">
         <v>128</v>
       </c>
-      <c r="F763">
+      <c r="F763" s="2">
         <v>6.6</v>
       </c>
-      <c r="G763">
+      <c r="G763" s="2">
         <v>9.6</v>
       </c>
-      <c r="H763">
+      <c r="H763" s="2">
         <v>5.3</v>
       </c>
-      <c r="I763">
+      <c r="I763" s="2">
         <v>5.3</v>
       </c>
-      <c r="J763">
+      <c r="J763" s="2">
         <v>2.7</v>
       </c>
     </row>
     <row r="764" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A764" s="29">
+      <c r="A764" s="16">
         <v>46031</v>
       </c>
-      <c r="B764" s="30">
+      <c r="B764" s="17">
         <v>0.47916666666666669</v>
       </c>
-      <c r="C764" t="s">
+      <c r="C764" s="2" t="s">
         <v>1124</v>
       </c>
-      <c r="D764" t="s">
+      <c r="D764" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E764">
+      <c r="E764" s="2">
         <v>155</v>
       </c>
-      <c r="F764">
+      <c r="F764" s="2">
         <v>15.5</v>
       </c>
-      <c r="G764">
+      <c r="G764" s="2">
         <v>15</v>
       </c>
-      <c r="H764">
-        <v>2</v>
-      </c>
-      <c r="I764">
+      <c r="H764" s="2">
+        <v>2</v>
+      </c>
+      <c r="I764" s="2">
         <v>7</v>
       </c>
-      <c r="J764">
+      <c r="J764" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="765" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A765" s="29">
+      <c r="A765" s="16">
         <v>46031</v>
       </c>
-      <c r="B765" s="30">
+      <c r="B765" s="17">
         <v>0.58333333333333337</v>
       </c>
-      <c r="C765" t="s">
+      <c r="C765" s="2" t="s">
         <v>1125</v>
       </c>
-      <c r="D765" t="s">
+      <c r="D765" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E765">
+      <c r="E765" s="2">
         <v>290</v>
       </c>
-      <c r="F765">
+      <c r="F765" s="2">
         <v>11</v>
       </c>
-      <c r="G765">
+      <c r="G765" s="2">
         <v>18</v>
       </c>
-      <c r="H765">
+      <c r="H765" s="2">
         <v>18</v>
       </c>
-      <c r="I765">
+      <c r="I765" s="2">
         <v>0</v>
       </c>
-      <c r="J765">
+      <c r="J765" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="766" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A766" s="29">
+      <c r="A766" s="16">
         <v>46031</v>
       </c>
-      <c r="B766" s="30">
+      <c r="B766" s="17">
         <v>0.75</v>
       </c>
-      <c r="C766" t="s">
+      <c r="C766" s="2" t="s">
         <v>1126</v>
       </c>
-      <c r="D766" t="s">
+      <c r="D766" s="2" t="s">
         <v>1127</v>
       </c>
-      <c r="E766">
+      <c r="E766" s="2">
         <v>400</v>
       </c>
-      <c r="F766">
+      <c r="F766" s="2">
         <v>25</v>
       </c>
-      <c r="G766">
+      <c r="G766" s="2">
         <v>40</v>
       </c>
-      <c r="H766">
+      <c r="H766" s="2">
         <v>15</v>
       </c>
-      <c r="I766">
+      <c r="I766" s="2">
         <v>5</v>
       </c>
-      <c r="J766">
+      <c r="J766" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="767" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A767" s="29">
+      <c r="A767" s="16">
         <v>46031</v>
       </c>
-      <c r="B767" s="30">
+      <c r="B767" s="17">
         <v>0.77083333333333337</v>
       </c>
-      <c r="C767" t="s">
+      <c r="C767" s="2" t="s">
         <v>1128</v>
       </c>
-      <c r="D767" t="s">
+      <c r="D767" s="2" t="s">
         <v>917</v>
       </c>
-      <c r="E767">
+      <c r="E767" s="2">
         <v>502.5</v>
       </c>
-      <c r="F767">
+      <c r="F767" s="2">
         <v>31.5</v>
       </c>
-      <c r="G767">
+      <c r="G767" s="2">
         <v>49.5</v>
       </c>
-      <c r="H767">
+      <c r="H767" s="2">
         <v>19.5</v>
       </c>
-      <c r="I767">
+      <c r="I767" s="2">
         <v>3.75</v>
       </c>
-      <c r="J767">
+      <c r="J767" s="2">
         <v>3.75</v>
       </c>
     </row>
     <row r="768" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A768" s="29">
+      <c r="A768" s="16">
         <v>46031</v>
       </c>
-      <c r="B768" s="30">
+      <c r="B768" s="17">
         <v>0.79166666666666663</v>
       </c>
-      <c r="C768" t="s">
+      <c r="C768" s="2" t="s">
         <v>1129</v>
       </c>
-      <c r="D768" t="s">
+      <c r="D768" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E768">
+      <c r="E768" s="2">
         <v>155</v>
       </c>
-      <c r="F768">
+      <c r="F768" s="2">
         <v>15.5</v>
       </c>
-      <c r="G768">
+      <c r="G768" s="2">
         <v>15</v>
       </c>
-      <c r="H768">
-        <v>2</v>
-      </c>
-      <c r="I768">
+      <c r="H768" s="2">
+        <v>2</v>
+      </c>
+      <c r="I768" s="2">
         <v>7</v>
       </c>
-      <c r="J768">
+      <c r="J768" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="769" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A769" s="29">
+      <c r="A769" s="16">
         <v>46032</v>
       </c>
-      <c r="B769" s="30">
+      <c r="B769" s="17">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C769" t="s">
+      <c r="C769" s="2" t="s">
         <v>1130</v>
       </c>
-      <c r="D769" t="s">
+      <c r="D769" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E769">
+      <c r="E769" s="2">
         <v>77</v>
       </c>
-      <c r="F769">
-        <v>2</v>
-      </c>
-      <c r="G769">
+      <c r="F769" s="2">
+        <v>2</v>
+      </c>
+      <c r="G769" s="2">
         <v>11</v>
       </c>
-      <c r="H769">
-        <v>2</v>
-      </c>
-      <c r="I769">
+      <c r="H769" s="2">
+        <v>2</v>
+      </c>
+      <c r="I769" s="2">
         <v>7</v>
       </c>
-      <c r="J769">
+      <c r="J769" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="770" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A770" s="29">
+      <c r="A770" s="16">
         <v>46032</v>
       </c>
-      <c r="B770" s="30">
+      <c r="B770" s="17">
         <v>0.35416666666666669</v>
       </c>
-      <c r="C770" t="s">
+      <c r="C770" s="2" t="s">
         <v>1131</v>
       </c>
-      <c r="D770" t="s">
+      <c r="D770" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E770">
+      <c r="E770" s="2">
         <v>128</v>
       </c>
-      <c r="F770">
+      <c r="F770" s="2">
         <v>6.6</v>
       </c>
-      <c r="G770">
+      <c r="G770" s="2">
         <v>9.6</v>
       </c>
-      <c r="H770">
+      <c r="H770" s="2">
         <v>5.3</v>
       </c>
-      <c r="I770">
+      <c r="I770" s="2">
         <v>5.3</v>
       </c>
-      <c r="J770">
+      <c r="J770" s="2">
         <v>2.7</v>
       </c>
     </row>
     <row r="771" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A771" s="29">
+      <c r="A771" s="16">
         <v>46032</v>
       </c>
-      <c r="B771" s="30">
+      <c r="B771" s="17">
         <v>0.58333333333333337</v>
       </c>
-      <c r="C771" t="s">
+      <c r="C771" s="2" t="s">
         <v>1132</v>
       </c>
-      <c r="D771" t="s">
+      <c r="D771" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E771">
+      <c r="E771" s="2">
         <v>290</v>
       </c>
-      <c r="F771">
+      <c r="F771" s="2">
         <v>11</v>
       </c>
-      <c r="G771">
+      <c r="G771" s="2">
         <v>18</v>
       </c>
-      <c r="H771">
+      <c r="H771" s="2">
         <v>18</v>
       </c>
-      <c r="I771">
+      <c r="I771" s="2">
         <v>0</v>
       </c>
-      <c r="J771">
+      <c r="J771" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="772" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A772" s="29">
+      <c r="A772" s="16">
         <v>46032</v>
       </c>
-      <c r="B772" s="30">
+      <c r="B772" s="17">
         <v>0.60416666666666663</v>
       </c>
-      <c r="C772" t="s">
+      <c r="C772" s="2" t="s">
         <v>1133</v>
       </c>
-      <c r="D772" t="s">
+      <c r="D772" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="E772">
+      <c r="E772" s="2">
         <v>78.75</v>
       </c>
-      <c r="F772">
+      <c r="F772" s="2">
         <v>1.95</v>
       </c>
-      <c r="G772">
+      <c r="G772" s="2">
         <v>16.8</v>
       </c>
-      <c r="H772">
+      <c r="H772" s="2">
         <v>0.55000000000000004</v>
       </c>
-      <c r="I772">
+      <c r="I772" s="2">
         <v>11.25</v>
       </c>
-      <c r="J772">
+      <c r="J772" s="2">
         <v>7.5</v>
       </c>
     </row>
     <row r="773" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A773" s="29">
+      <c r="A773" s="16">
         <v>46032</v>
       </c>
-      <c r="B773" s="30">
+      <c r="B773" s="17">
         <v>0.625</v>
       </c>
-      <c r="C773" t="s">
+      <c r="C773" s="2" t="s">
         <v>1134</v>
       </c>
-      <c r="D773" t="s">
+      <c r="D773" s="2" t="s">
         <v>1114</v>
       </c>
-      <c r="E773">
+      <c r="E773" s="2">
         <v>82.5</v>
       </c>
-      <c r="F773">
+      <c r="F773" s="2">
         <v>2.5</v>
       </c>
-      <c r="G773">
+      <c r="G773" s="2">
         <v>4.5</v>
       </c>
-      <c r="H773">
+      <c r="H773" s="2">
         <v>6.75</v>
       </c>
-      <c r="I773">
+      <c r="I773" s="2">
         <v>0.75</v>
       </c>
-      <c r="J773">
+      <c r="J773" s="2">
         <v>0.5</v>
       </c>
     </row>
     <row r="774" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A774" s="29">
+      <c r="A774" s="16">
         <v>46032</v>
       </c>
-      <c r="B774" s="30">
+      <c r="B774" s="17">
         <v>0.6875</v>
       </c>
-      <c r="C774" t="s">
+      <c r="C774" s="2" t="s">
         <v>1135</v>
       </c>
-      <c r="D774" t="s">
+      <c r="D774" s="2" t="s">
         <v>932</v>
       </c>
-      <c r="E774">
+      <c r="E774" s="2">
         <v>335</v>
       </c>
-      <c r="F774">
+      <c r="F774" s="2">
         <v>21</v>
       </c>
-      <c r="G774">
+      <c r="G774" s="2">
         <v>33</v>
       </c>
-      <c r="H774">
+      <c r="H774" s="2">
         <v>13</v>
       </c>
-      <c r="I774">
+      <c r="I774" s="2">
         <v>2.5</v>
       </c>
-      <c r="J774">
+      <c r="J774" s="2">
         <v>2.5</v>
       </c>
     </row>
     <row r="775" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A775" s="29">
+      <c r="A775" s="16">
         <v>46032</v>
       </c>
-      <c r="B775" s="30">
+      <c r="B775" s="17">
         <v>0.70833333333333337</v>
       </c>
-      <c r="C775" t="s">
+      <c r="C775" s="2" t="s">
         <v>1136</v>
       </c>
-      <c r="D775" t="s">
+      <c r="D775" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E775">
+      <c r="E775" s="2">
         <v>155</v>
       </c>
-      <c r="F775">
+      <c r="F775" s="2">
         <v>15.5</v>
       </c>
-      <c r="G775">
+      <c r="G775" s="2">
         <v>15</v>
       </c>
-      <c r="H775">
-        <v>2</v>
-      </c>
-      <c r="I775">
+      <c r="H775" s="2">
+        <v>2</v>
+      </c>
+      <c r="I775" s="2">
         <v>7</v>
       </c>
-      <c r="J775">
+      <c r="J775" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="776" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A776" s="29">
+      <c r="A776" s="16">
         <v>46032</v>
       </c>
-      <c r="B776" s="30">
+      <c r="B776" s="17">
         <v>0.8125</v>
       </c>
-      <c r="C776" t="s">
+      <c r="C776" s="2" t="s">
         <v>1137</v>
       </c>
-      <c r="D776" t="s">
+      <c r="D776" s="2" t="s">
         <v>1138</v>
       </c>
-      <c r="E776">
+      <c r="E776" s="2">
         <v>460</v>
       </c>
-      <c r="F776">
+      <c r="F776" s="2">
         <v>30</v>
       </c>
-      <c r="G776">
+      <c r="G776" s="2">
         <v>50</v>
       </c>
-      <c r="H776">
+      <c r="H776" s="2">
         <v>15</v>
       </c>
-      <c r="I776">
-        <v>2</v>
-      </c>
-      <c r="J776">
+      <c r="I776" s="2">
+        <v>2</v>
+      </c>
+      <c r="J776" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="777" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A777" s="29">
+      <c r="A777" s="16">
         <v>46033</v>
       </c>
-      <c r="B777" s="30">
+      <c r="B777" s="17">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C777" t="s">
+      <c r="C777" s="2" t="s">
         <v>1145</v>
       </c>
-      <c r="D777" t="s">
+      <c r="D777" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E777">
+      <c r="E777" s="2">
         <v>77</v>
       </c>
-      <c r="F777">
-        <v>2</v>
-      </c>
-      <c r="G777">
+      <c r="F777" s="2">
+        <v>2</v>
+      </c>
+      <c r="G777" s="2">
         <v>11</v>
       </c>
-      <c r="H777">
-        <v>2</v>
-      </c>
-      <c r="I777">
+      <c r="H777" s="2">
+        <v>2</v>
+      </c>
+      <c r="I777" s="2">
         <v>7</v>
       </c>
-      <c r="J777">
+      <c r="J777" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="778" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A778" s="29">
+      <c r="A778" s="16">
         <v>46033</v>
       </c>
-      <c r="B778" s="30">
+      <c r="B778" s="17">
         <v>0.35416666666666669</v>
       </c>
-      <c r="C778" t="s">
+      <c r="C778" s="2" t="s">
         <v>1146</v>
       </c>
-      <c r="D778" t="s">
+      <c r="D778" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E778">
+      <c r="E778" s="2">
         <v>128</v>
       </c>
-      <c r="F778">
+      <c r="F778" s="2">
         <v>6.6</v>
       </c>
-      <c r="G778">
+      <c r="G778" s="2">
         <v>9.6</v>
       </c>
-      <c r="H778">
+      <c r="H778" s="2">
         <v>5.3</v>
       </c>
-      <c r="I778">
+      <c r="I778" s="2">
         <v>5.3</v>
       </c>
-      <c r="J778">
+      <c r="J778" s="2">
         <v>2.7</v>
       </c>
     </row>
     <row r="779" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A779" s="29">
+      <c r="A779" s="16">
         <v>46033</v>
       </c>
-      <c r="B779" s="30">
+      <c r="B779" s="17">
         <v>0.41666666666666669</v>
       </c>
-      <c r="C779" t="s">
+      <c r="C779" s="2" t="s">
         <v>1147</v>
       </c>
-      <c r="D779" t="s">
+      <c r="D779" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="E779">
+      <c r="E779" s="2">
         <v>78.75</v>
       </c>
-      <c r="F779">
+      <c r="F779" s="2">
         <v>1.95</v>
       </c>
-      <c r="G779">
+      <c r="G779" s="2">
         <v>16.8</v>
       </c>
-      <c r="H779">
+      <c r="H779" s="2">
         <v>0.55000000000000004</v>
       </c>
-      <c r="I779">
+      <c r="I779" s="2">
         <v>11.25</v>
       </c>
-      <c r="J779">
+      <c r="J779" s="2">
         <v>7.5</v>
       </c>
     </row>
     <row r="780" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A780" s="29">
+      <c r="A780" s="16">
         <v>46033</v>
       </c>
-      <c r="B780" s="30">
+      <c r="B780" s="17">
         <v>0.5</v>
       </c>
-      <c r="C780" t="s">
+      <c r="C780" s="2" t="s">
         <v>1148</v>
       </c>
-      <c r="D780" t="s">
+      <c r="D780" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E780">
+      <c r="E780" s="2">
         <v>290</v>
       </c>
-      <c r="F780">
+      <c r="F780" s="2">
         <v>11</v>
       </c>
-      <c r="G780">
+      <c r="G780" s="2">
         <v>18</v>
       </c>
-      <c r="H780">
+      <c r="H780" s="2">
         <v>18</v>
       </c>
-      <c r="I780">
+      <c r="I780" s="2">
         <v>0</v>
       </c>
-      <c r="J780">
+      <c r="J780" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="781" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A781" s="29">
+      <c r="A781" s="16">
         <v>46033</v>
       </c>
-      <c r="B781" s="30">
+      <c r="B781" s="17">
         <v>0.52083333333333337</v>
       </c>
-      <c r="C781" t="s">
+      <c r="C781" s="2" t="s">
         <v>1149</v>
       </c>
-      <c r="D781" t="s">
+      <c r="D781" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E781">
+      <c r="E781" s="2">
         <v>175</v>
       </c>
-      <c r="F781">
+      <c r="F781" s="2">
         <v>15.5</v>
       </c>
-      <c r="G781">
+      <c r="G781" s="2">
         <v>20</v>
       </c>
-      <c r="H781">
-        <v>2</v>
-      </c>
-      <c r="I781">
+      <c r="H781" s="2">
+        <v>2</v>
+      </c>
+      <c r="I781" s="2">
         <v>11.5</v>
       </c>
-      <c r="J781">
+      <c r="J781" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="782" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A782" s="29">
+      <c r="A782" s="16">
         <v>46033</v>
       </c>
-      <c r="B782" s="30">
+      <c r="B782" s="17">
         <v>0.5625</v>
       </c>
-      <c r="C782" t="s">
+      <c r="C782" s="2" t="s">
         <v>1150</v>
       </c>
-      <c r="D782" t="s">
+      <c r="D782" s="2" t="s">
         <v>1151</v>
       </c>
-      <c r="E782">
+      <c r="E782" s="2">
         <v>330</v>
       </c>
-      <c r="F782">
+      <c r="F782" s="2">
         <v>20</v>
       </c>
-      <c r="G782">
+      <c r="G782" s="2">
         <v>50</v>
       </c>
-      <c r="H782">
+      <c r="H782" s="2">
         <v>8</v>
       </c>
-      <c r="I782">
-        <v>2</v>
-      </c>
-      <c r="J782">
+      <c r="I782" s="2">
+        <v>2</v>
+      </c>
+      <c r="J782" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="783" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A783" s="29">
+      <c r="A783" s="16">
         <v>46033</v>
       </c>
-      <c r="B783" s="30">
+      <c r="B783" s="17">
         <v>0.66666666666666663</v>
       </c>
-      <c r="C783" t="s">
+      <c r="C783" s="2" t="s">
         <v>1152</v>
       </c>
-      <c r="D783" t="s">
+      <c r="D783" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E783">
+      <c r="E783" s="2">
         <v>77</v>
       </c>
-      <c r="F783">
-        <v>2</v>
-      </c>
-      <c r="G783">
+      <c r="F783" s="2">
+        <v>2</v>
+      </c>
+      <c r="G783" s="2">
         <v>11</v>
       </c>
-      <c r="H783">
-        <v>2</v>
-      </c>
-      <c r="I783">
+      <c r="H783" s="2">
+        <v>2</v>
+      </c>
+      <c r="I783" s="2">
         <v>7</v>
       </c>
-      <c r="J783">
+      <c r="J783" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="784" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A784" s="29">
+      <c r="A784" s="16">
         <v>46033</v>
       </c>
-      <c r="B784" s="30">
+      <c r="B784" s="17">
         <v>0.6875</v>
       </c>
-      <c r="C784" t="s">
+      <c r="C784" s="2" t="s">
         <v>1153</v>
       </c>
-      <c r="D784" t="s">
+      <c r="D784" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="E784">
+      <c r="E784" s="2">
         <v>44.5</v>
       </c>
-      <c r="F784">
+      <c r="F784" s="2">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G784">
+      <c r="G784" s="2">
         <v>11.5</v>
       </c>
-      <c r="H784">
+      <c r="H784" s="2">
         <v>0.15</v>
       </c>
-      <c r="I784">
+      <c r="I784" s="2">
         <v>6</v>
       </c>
-      <c r="J784">
+      <c r="J784" s="2">
         <v>1.3</v>
       </c>
     </row>
     <row r="785" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A785" s="29">
+      <c r="A785" s="16">
         <v>46033</v>
       </c>
-      <c r="B785" s="30">
+      <c r="B785" s="17">
         <v>0.70833333333333337</v>
       </c>
-      <c r="C785" t="s">
+      <c r="C785" s="2" t="s">
         <v>1154</v>
       </c>
-      <c r="D785" t="s">
+      <c r="D785" s="2" t="s">
         <v>1114</v>
       </c>
-      <c r="E785">
+      <c r="E785" s="2">
         <v>82.5</v>
       </c>
-      <c r="F785">
+      <c r="F785" s="2">
         <v>2.5</v>
       </c>
-      <c r="G785">
+      <c r="G785" s="2">
         <v>4.5</v>
       </c>
-      <c r="H785">
+      <c r="H785" s="2">
         <v>6.75</v>
       </c>
-      <c r="I785">
+      <c r="I785" s="2">
         <v>0.75</v>
       </c>
-      <c r="J785">
+      <c r="J785" s="2">
         <v>0.5</v>
       </c>
     </row>
     <row r="786" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A786" s="29">
+      <c r="A786" s="16">
         <v>46033</v>
       </c>
-      <c r="B786" s="30">
+      <c r="B786" s="17">
         <v>0.77083333333333337</v>
       </c>
-      <c r="C786" t="s">
+      <c r="C786" s="2" t="s">
         <v>1155</v>
       </c>
-      <c r="D786" t="s">
+      <c r="D786" s="2" t="s">
         <v>932</v>
       </c>
-      <c r="E786">
+      <c r="E786" s="2">
         <v>335</v>
       </c>
-      <c r="F786">
+      <c r="F786" s="2">
         <v>21</v>
       </c>
-      <c r="G786">
+      <c r="G786" s="2">
         <v>33</v>
       </c>
-      <c r="H786">
+      <c r="H786" s="2">
         <v>13</v>
       </c>
-      <c r="I786">
+      <c r="I786" s="2">
         <v>2.5</v>
       </c>
-      <c r="J786">
+      <c r="J786" s="2">
         <v>2.5</v>
       </c>
     </row>
     <row r="787" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A787" s="29">
+      <c r="A787" s="16">
         <v>46033</v>
       </c>
-      <c r="B787" s="30">
+      <c r="B787" s="17">
         <v>0.83333333333333337</v>
       </c>
-      <c r="C787" t="s">
+      <c r="C787" s="2" t="s">
         <v>1156</v>
       </c>
-      <c r="D787" t="s">
+      <c r="D787" s="2" t="s">
         <v>1157</v>
       </c>
-      <c r="E787">
+      <c r="E787" s="2">
         <v>78</v>
       </c>
-      <c r="F787">
+      <c r="F787" s="2">
         <v>0.6</v>
       </c>
-      <c r="G787">
+      <c r="G787" s="2">
         <v>20.8</v>
       </c>
-      <c r="H787">
+      <c r="H787" s="2">
         <v>0.2</v>
       </c>
-      <c r="I787">
+      <c r="I787" s="2">
         <v>16.100000000000001</v>
       </c>
-      <c r="J787">
+      <c r="J787" s="2">
         <v>3.5</v>
       </c>
     </row>
     <row r="788" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A788" s="29">
+      <c r="A788" s="16">
         <v>46033</v>
       </c>
-      <c r="B788" s="30">
+      <c r="B788" s="17">
         <v>0.85416666666666663</v>
       </c>
-      <c r="C788" t="s">
+      <c r="C788" s="2" t="s">
         <v>1158</v>
       </c>
-      <c r="D788" t="s">
+      <c r="D788" s="2" t="s">
         <v>1159</v>
       </c>
-      <c r="E788">
+      <c r="E788" s="2">
         <v>300</v>
       </c>
-      <c r="F788">
+      <c r="F788" s="2">
         <v>18</v>
       </c>
-      <c r="G788">
+      <c r="G788" s="2">
         <v>20</v>
       </c>
-      <c r="H788">
+      <c r="H788" s="2">
         <v>18</v>
       </c>
-      <c r="I788">
-        <v>2</v>
-      </c>
-      <c r="J788">
+      <c r="I788" s="2">
+        <v>2</v>
+      </c>
+      <c r="J788" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="789" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A789" s="29">
+      <c r="A789" s="16">
         <v>46034</v>
       </c>
-      <c r="B789" s="30">
+      <c r="B789" s="17">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C789" t="s">
+      <c r="C789" s="2" t="s">
         <v>1160</v>
       </c>
-      <c r="D789" t="s">
+      <c r="D789" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E789">
+      <c r="E789" s="2">
         <v>77</v>
       </c>
-      <c r="F789">
-        <v>2</v>
-      </c>
-      <c r="G789">
+      <c r="F789" s="2">
+        <v>2</v>
+      </c>
+      <c r="G789" s="2">
         <v>11</v>
       </c>
-      <c r="H789">
-        <v>2</v>
-      </c>
-      <c r="I789">
+      <c r="H789" s="2">
+        <v>2</v>
+      </c>
+      <c r="I789" s="2">
         <v>7</v>
       </c>
-      <c r="J789">
+      <c r="J789" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="790" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A790" s="29">
+      <c r="A790" s="16">
         <v>46034</v>
       </c>
-      <c r="B790" s="30">
+      <c r="B790" s="17">
         <v>0.35416666666666669</v>
       </c>
-      <c r="C790" t="s">
+      <c r="C790" s="2" t="s">
         <v>1161</v>
       </c>
-      <c r="D790" t="s">
+      <c r="D790" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E790">
+      <c r="E790" s="2">
         <v>128</v>
       </c>
-      <c r="F790">
+      <c r="F790" s="2">
         <v>6.6</v>
       </c>
-      <c r="G790">
+      <c r="G790" s="2">
         <v>9.6</v>
       </c>
-      <c r="H790">
+      <c r="H790" s="2">
         <v>5.3</v>
       </c>
-      <c r="I790">
+      <c r="I790" s="2">
         <v>5.3</v>
       </c>
-      <c r="J790">
+      <c r="J790" s="2">
         <v>2.7</v>
       </c>
     </row>
     <row r="791" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A791" s="29">
+      <c r="A791" s="16">
         <v>46034</v>
       </c>
-      <c r="B791" s="30">
+      <c r="B791" s="17">
         <v>0.375</v>
       </c>
-      <c r="C791" t="s">
+      <c r="C791" s="2" t="s">
         <v>1162</v>
       </c>
-      <c r="D791" t="s">
+      <c r="D791" s="2" t="s">
         <v>1114</v>
       </c>
-      <c r="E791">
+      <c r="E791" s="2">
         <v>82.5</v>
       </c>
-      <c r="F791">
+      <c r="F791" s="2">
         <v>2.5</v>
       </c>
-      <c r="G791">
+      <c r="G791" s="2">
         <v>4.5</v>
       </c>
-      <c r="H791">
+      <c r="H791" s="2">
         <v>6.75</v>
       </c>
-      <c r="I791">
+      <c r="I791" s="2">
         <v>0.75</v>
       </c>
-      <c r="J791">
+      <c r="J791" s="2">
         <v>0.5</v>
       </c>
     </row>
     <row r="792" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A792" s="29">
+      <c r="A792" s="16">
         <v>46034</v>
       </c>
-      <c r="B792" s="30">
+      <c r="B792" s="17">
         <v>0.5</v>
       </c>
-      <c r="C792" t="s">
+      <c r="C792" s="2" t="s">
         <v>1163</v>
       </c>
-      <c r="D792" t="s">
+      <c r="D792" s="2" t="s">
         <v>1164</v>
       </c>
-      <c r="E792">
+      <c r="E792" s="2">
         <v>340</v>
       </c>
-      <c r="F792">
+      <c r="F792" s="2">
         <v>18</v>
       </c>
-      <c r="G792">
+      <c r="G792" s="2">
         <v>30</v>
       </c>
-      <c r="H792">
+      <c r="H792" s="2">
         <v>17</v>
       </c>
-      <c r="I792">
-        <v>2</v>
-      </c>
-      <c r="J792">
+      <c r="I792" s="2">
+        <v>2</v>
+      </c>
+      <c r="J792" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="793" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A793" s="29">
+      <c r="A793" s="16">
         <v>46034</v>
       </c>
-      <c r="B793" s="30">
+      <c r="B793" s="17">
         <v>0.70833333333333337</v>
       </c>
-      <c r="C793" t="s">
+      <c r="C793" s="2" t="s">
         <v>1165</v>
       </c>
-      <c r="D793" t="s">
+      <c r="D793" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E793">
+      <c r="E793" s="2">
         <v>77</v>
       </c>
-      <c r="F793">
-        <v>2</v>
-      </c>
-      <c r="G793">
+      <c r="F793" s="2">
+        <v>2</v>
+      </c>
+      <c r="G793" s="2">
         <v>11</v>
       </c>
-      <c r="H793">
-        <v>2</v>
-      </c>
-      <c r="I793">
+      <c r="H793" s="2">
+        <v>2</v>
+      </c>
+      <c r="I793" s="2">
         <v>7</v>
       </c>
-      <c r="J793">
+      <c r="J793" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="794" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A794" s="29">
+      <c r="A794" s="16">
         <v>46034</v>
       </c>
-      <c r="B794" s="30">
+      <c r="B794" s="17">
         <v>0.77083333333333337</v>
       </c>
-      <c r="C794" t="s">
+      <c r="C794" s="2" t="s">
         <v>1166</v>
       </c>
-      <c r="D794" t="s">
+      <c r="D794" s="2" t="s">
         <v>1167</v>
       </c>
-      <c r="E794">
+      <c r="E794" s="2">
         <v>343</v>
       </c>
-      <c r="F794">
+      <c r="F794" s="2">
         <v>20</v>
       </c>
-      <c r="G794">
+      <c r="G794" s="2">
         <v>35</v>
       </c>
-      <c r="H794">
+      <c r="H794" s="2">
         <v>15</v>
       </c>
-      <c r="I794">
+      <c r="I794" s="2">
         <v>5</v>
       </c>
-      <c r="J794">
+      <c r="J794" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="795" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A795" s="29">
+      <c r="A795" s="16">
         <v>46034</v>
       </c>
-      <c r="B795" s="30">
+      <c r="B795" s="17">
         <v>0.79166666666666663</v>
       </c>
-      <c r="C795" t="s">
+      <c r="C795" s="2" t="s">
         <v>1168</v>
       </c>
-      <c r="D795" t="s">
+      <c r="D795" s="2" t="s">
         <v>932</v>
       </c>
-      <c r="E795">
+      <c r="E795" s="2">
         <v>335</v>
       </c>
-      <c r="F795">
+      <c r="F795" s="2">
         <v>21</v>
       </c>
-      <c r="G795">
+      <c r="G795" s="2">
         <v>33</v>
       </c>
-      <c r="H795">
+      <c r="H795" s="2">
         <v>13</v>
       </c>
-      <c r="I795">
+      <c r="I795" s="2">
         <v>2.5</v>
       </c>
-      <c r="J795">
+      <c r="J795" s="2">
         <v>2.5</v>
       </c>
     </row>
     <row r="796" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A796" s="29">
+      <c r="A796" s="16">
         <v>46034</v>
       </c>
-      <c r="B796" s="30">
+      <c r="B796" s="17">
         <v>0.8125</v>
       </c>
-      <c r="C796" t="s">
+      <c r="C796" s="2" t="s">
         <v>1169</v>
       </c>
-      <c r="D796" t="s">
+      <c r="D796" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E796">
+      <c r="E796" s="2">
         <v>175</v>
       </c>
-      <c r="F796">
+      <c r="F796" s="2">
         <v>15.5</v>
       </c>
-      <c r="G796">
+      <c r="G796" s="2">
         <v>20</v>
       </c>
-      <c r="H796">
-        <v>2</v>
-      </c>
-      <c r="I796">
+      <c r="H796" s="2">
+        <v>2</v>
+      </c>
+      <c r="I796" s="2">
         <v>11.5</v>
       </c>
-      <c r="J796">
+      <c r="J796" s="2">
         <v>1.8</v>
       </c>
     </row>
     <row r="797" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A797" s="29">
+      <c r="A797" s="16">
         <v>46035</v>
       </c>
-      <c r="B797" s="30">
+      <c r="B797" s="17">
         <v>0.33333333333333331</v>
       </c>
-      <c r="C797" t="s">
+      <c r="C797" s="2" t="s">
         <v>1170</v>
       </c>
-      <c r="D797" t="s">
+      <c r="D797" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E797">
+      <c r="E797" s="2">
         <v>77</v>
       </c>
-      <c r="F797">
-        <v>2</v>
-      </c>
-      <c r="G797">
+      <c r="F797" s="2">
+        <v>2</v>
+      </c>
+      <c r="G797" s="2">
         <v>11</v>
       </c>
-      <c r="H797">
-        <v>2</v>
-      </c>
-      <c r="I797">
+      <c r="H797" s="2">
+        <v>2</v>
+      </c>
+      <c r="I797" s="2">
         <v>7</v>
       </c>
-      <c r="J797">
+      <c r="J797" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="798" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A798" s="29">
+      <c r="A798" s="16">
         <v>46035</v>
       </c>
-      <c r="B798" s="30">
+      <c r="B798" s="17">
         <v>0.35416666666666669</v>
       </c>
-      <c r="C798" t="s">
+      <c r="C798" s="2" t="s">
         <v>1171</v>
       </c>
-      <c r="D798" t="s">
+      <c r="D798" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E798">
+      <c r="E798" s="2">
         <v>128</v>
       </c>
-      <c r="F798">
+      <c r="F798" s="2">
         <v>6.6</v>
       </c>
-      <c r="G798">
+      <c r="G798" s="2">
         <v>9.6</v>
       </c>
-      <c r="H798">
+      <c r="H798" s="2">
         <v>5.3</v>
       </c>
-      <c r="I798">
+      <c r="I798" s="2">
         <v>5.3</v>
       </c>
-      <c r="J798">
+      <c r="J798" s="2">
         <v>2.7</v>
       </c>
     </row>
     <row r="799" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A799" s="29">
+      <c r="A799" s="16">
         <v>46035</v>
       </c>
-      <c r="B799" s="30">
+      <c r="B799" s="17">
         <v>0.375</v>
       </c>
-      <c r="C799" t="s">
+      <c r="C799" s="2" t="s">
         <v>1172</v>
       </c>
-      <c r="D799" t="s">
+      <c r="D799" s="2" t="s">
         <v>1114</v>
       </c>
-      <c r="E799">
+      <c r="E799" s="2">
         <v>82.5</v>
       </c>
-      <c r="F799">
+      <c r="F799" s="2">
         <v>2.5</v>
       </c>
-      <c r="G799">
+      <c r="G799" s="2">
         <v>4.5</v>
       </c>
-      <c r="H799">
+      <c r="H799" s="2">
         <v>6.75</v>
       </c>
-      <c r="I799">
+      <c r="I799" s="2">
         <v>0.75</v>
       </c>
-      <c r="J799">
+      <c r="J799" s="2">
         <v>0.5</v>
       </c>
     </row>
     <row r="800" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A800" s="29">
+      <c r="A800" s="16">
         <v>46035</v>
       </c>
-      <c r="B800" s="30">
+      <c r="B800" s="17">
         <v>0.39583333333333331</v>
       </c>
-      <c r="C800" t="s">
+      <c r="C800" s="2" t="s">
         <v>1173</v>
       </c>
-      <c r="D800" t="s">
+      <c r="D800" s="2" t="s">
         <v>1157</v>
       </c>
-      <c r="E800">
+      <c r="E800" s="2">
         <v>78</v>
       </c>
-      <c r="F800">
+      <c r="F800" s="2">
         <v>0.6</v>
       </c>
-      <c r="G800">
+      <c r="G800" s="2">
         <v>20.8</v>
       </c>
-      <c r="H800">
+      <c r="H800" s="2">
         <v>0.2</v>
       </c>
-      <c r="I800">
+      <c r="I800" s="2">
         <v>16.100000000000001</v>
       </c>
-      <c r="J800">
+      <c r="J800" s="2">
         <v>3.5</v>
       </c>
     </row>
     <row r="801" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A801" s="29">
+      <c r="A801" s="16">
         <v>46035</v>
       </c>
-      <c r="B801" s="30">
+      <c r="B801" s="17">
         <v>0.41666666666666669</v>
       </c>
-      <c r="C801" t="s">
+      <c r="C801" s="2" t="s">
         <v>1174</v>
       </c>
-      <c r="D801" t="s">
+      <c r="D801" s="2" t="s">
         <v>1175</v>
       </c>
-      <c r="E801">
+      <c r="E801" s="2">
         <v>240</v>
       </c>
-      <c r="F801">
+      <c r="F801" s="2">
         <v>6</v>
       </c>
-      <c r="G801">
+      <c r="G801" s="2">
         <v>40</v>
       </c>
-      <c r="H801">
+      <c r="H801" s="2">
         <v>6</v>
       </c>
-      <c r="I801">
+      <c r="I801" s="2">
         <v>8</v>
       </c>
-      <c r="J801">
+      <c r="J801" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="802" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A802" s="29">
+      <c r="A802" s="16">
         <v>46035</v>
       </c>
-      <c r="B802" s="30">
+      <c r="B802" s="17">
         <v>0.52083333333333337</v>
       </c>
-      <c r="C802" t="s">
+      <c r="C802" s="2" t="s">
         <v>1176</v>
       </c>
-      <c r="D802" t="s">
+      <c r="D802" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E802">
+      <c r="E802" s="2">
         <v>290</v>
       </c>
-      <c r="F802">
+      <c r="F802" s="2">
         <v>11</v>
       </c>
-      <c r="G802">
+      <c r="G802" s="2">
         <v>18</v>
       </c>
-      <c r="H802">
+      <c r="H802" s="2">
         <v>18</v>
       </c>
-      <c r="I802">
+      <c r="I802" s="2">
         <v>0</v>
       </c>
-      <c r="J802">
+      <c r="J802" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="803" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A803" s="29">
+      <c r="A803" s="16">
         <v>46035</v>
       </c>
-      <c r="B803" s="30">
+      <c r="B803" s="17">
         <v>0.70833333333333337</v>
       </c>
-      <c r="C803" t="s">
+      <c r="C803" s="2" t="s">
         <v>1177</v>
       </c>
-      <c r="D803" t="s">
+      <c r="D803" s="2" t="s">
         <v>808</v>
       </c>
-      <c r="E803">
+      <c r="E803" s="2">
         <v>145</v>
       </c>
-      <c r="F803">
+      <c r="F803" s="2">
         <v>5.5</v>
       </c>
-      <c r="G803">
+      <c r="G803" s="2">
         <v>9</v>
       </c>
-      <c r="H803">
+      <c r="H803" s="2">
         <v>9</v>
       </c>
-      <c r="I803">
+      <c r="I803" s="2">
         <v>0</v>
       </c>
-      <c r="J803">
+      <c r="J803" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="804" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A804" s="29">
+      <c r="A804" s="16">
         <v>46035</v>
       </c>
-      <c r="B804" s="30">
+      <c r="B804" s="17">
         <v>0.72916666666666663</v>
       </c>
-      <c r="C804" t="s">
+      <c r="C804" s="2" t="s">
         <v>1178</v>
       </c>
-      <c r="D804" t="s">
+      <c r="D804" s="2" t="s">
         <v>932</v>
       </c>
-      <c r="E804">
+      <c r="E804" s="2">
         <v>335</v>
       </c>
-      <c r="F804">
+      <c r="F804" s="2">
         <v>21</v>
       </c>
-      <c r="G804">
+      <c r="G804" s="2">
         <v>33</v>
       </c>
-      <c r="H804">
+      <c r="H804" s="2">
         <v>13</v>
       </c>
-      <c r="I804">
+      <c r="I804" s="2">
         <v>2.5</v>
       </c>
-      <c r="J804">
+      <c r="J804" s="2">
         <v>2.5</v>
       </c>
     </row>
     <row r="805" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A805" s="29">
+      <c r="A805" s="16">
         <v>46035</v>
       </c>
-      <c r="B805" s="30">
+      <c r="B805" s="17">
         <v>0.75</v>
       </c>
-      <c r="C805" t="s">
+      <c r="C805" s="2" t="s">
         <v>1179</v>
       </c>
-      <c r="D805" t="s">
+      <c r="D805" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E805">
+      <c r="E805" s="2">
         <v>175</v>
       </c>
-      <c r="F805">
+      <c r="F805" s="2">
         <v>15.5</v>
       </c>
-      <c r="G805">
+      <c r="G805" s="2">
         <v>20</v>
       </c>
-      <c r="H805">
-        <v>2</v>
-      </c>
-      <c r="I805">
+      <c r="H805" s="2">
+        <v>2</v>
+      </c>
+      <c r="I805" s="2">
         <v>11.5</v>
       </c>
-      <c r="J805">
+      <c r="J805" s="2">
         <v>1.8</v>
+      </c>
+    </row>
+    <row r="806" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A806" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B806" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C806" s="2" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D806" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E806" s="2">
+        <v>77</v>
+      </c>
+      <c r="F806" s="2">
+        <v>2</v>
+      </c>
+      <c r="G806" s="2">
+        <v>11</v>
+      </c>
+      <c r="H806" s="2">
+        <v>2</v>
+      </c>
+      <c r="I806" s="2">
+        <v>7</v>
+      </c>
+      <c r="J806" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="807" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A807" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B807" s="17">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="C807" s="2" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D807" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E807" s="2">
+        <v>256</v>
+      </c>
+      <c r="F807" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="G807" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="H807" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="I807" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="J807" s="2">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="808" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A808" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B808" s="17">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="C808" s="2" t="s">
+        <v>1187</v>
+      </c>
+      <c r="D808" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E808" s="2">
+        <v>290</v>
+      </c>
+      <c r="F808" s="2">
+        <v>11</v>
+      </c>
+      <c r="G808" s="2">
+        <v>18</v>
+      </c>
+      <c r="H808" s="2">
+        <v>18</v>
+      </c>
+      <c r="I808" s="2">
+        <v>0</v>
+      </c>
+      <c r="J808" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="809" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A809" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B809" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="C809" s="2" t="s">
+        <v>1188</v>
+      </c>
+      <c r="D809" s="2" t="s">
+        <v>917</v>
+      </c>
+      <c r="E809" s="2">
+        <v>503</v>
+      </c>
+      <c r="F809" s="2">
+        <v>31.5</v>
+      </c>
+      <c r="G809" s="2">
+        <v>49.5</v>
+      </c>
+      <c r="H809" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="I809" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="J809" s="2">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="810" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A810" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B810" s="17">
+        <v>0.625</v>
+      </c>
+      <c r="C810" s="2" t="s">
+        <v>1189</v>
+      </c>
+      <c r="D810" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E810" s="2">
+        <v>156</v>
+      </c>
+      <c r="F810" s="2">
+        <v>12.6</v>
+      </c>
+      <c r="G810" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="H810" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="I810" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="J810" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="811" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A811" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B811" s="17">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="C811" s="2" t="s">
+        <v>1191</v>
+      </c>
+      <c r="D811" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E811" s="2">
+        <v>77</v>
+      </c>
+      <c r="F811" s="2">
+        <v>2</v>
+      </c>
+      <c r="G811" s="2">
+        <v>11</v>
+      </c>
+      <c r="H811" s="2">
+        <v>2</v>
+      </c>
+      <c r="I811" s="2">
+        <v>7</v>
+      </c>
+      <c r="J811" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="812" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A812" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B812" s="17">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C812" s="2" t="s">
+        <v>1192</v>
+      </c>
+      <c r="D812" s="2" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E812" s="2">
+        <v>89</v>
+      </c>
+      <c r="F812" s="2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G812" s="2">
+        <v>23</v>
+      </c>
+      <c r="H812" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="I812" s="2">
+        <v>12</v>
+      </c>
+      <c r="J812" s="2">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="813" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A813" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B813" s="17">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="C813" s="2" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D813" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E813" s="2">
+        <v>155</v>
+      </c>
+      <c r="F813" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G813" s="2">
+        <v>15</v>
+      </c>
+      <c r="H813" s="2">
+        <v>2</v>
+      </c>
+      <c r="I813" s="2">
+        <v>7</v>
+      </c>
+      <c r="J813" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="814" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A814" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B814" s="17">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="C814" s="2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D814" s="2" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E814" s="2">
+        <v>243</v>
+      </c>
+      <c r="F814" s="2">
+        <v>12</v>
+      </c>
+      <c r="G814" s="2">
+        <v>19</v>
+      </c>
+      <c r="H814" s="2">
+        <v>13</v>
+      </c>
+      <c r="I814" s="2">
+        <v>5</v>
+      </c>
+      <c r="J814" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="815" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A815" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B815" s="17">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C815" s="2" t="s">
+        <v>1197</v>
+      </c>
+      <c r="D815" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="E815" s="2">
+        <v>270</v>
+      </c>
+      <c r="F815" s="2">
+        <v>6</v>
+      </c>
+      <c r="G815" s="2">
+        <v>35</v>
+      </c>
+      <c r="H815" s="2">
+        <v>12</v>
+      </c>
+      <c r="I815" s="2">
+        <v>1</v>
+      </c>
+      <c r="J815" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="816" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A816" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B816" s="17">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C816" s="2" t="s">
+        <v>1198</v>
+      </c>
+      <c r="D816" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E816" s="2">
+        <v>128</v>
+      </c>
+      <c r="F816" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="G816" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="H816" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="I816" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J816" s="2">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="817" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A817" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B817" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C817" s="2" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D817" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E817" s="2">
+        <v>77</v>
+      </c>
+      <c r="F817" s="2">
+        <v>2</v>
+      </c>
+      <c r="G817" s="2">
+        <v>11</v>
+      </c>
+      <c r="H817" s="2">
+        <v>2</v>
+      </c>
+      <c r="I817" s="2">
+        <v>7</v>
+      </c>
+      <c r="J817" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="818" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A818" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B818" s="17">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="C818" s="2" t="s">
+        <v>1200</v>
+      </c>
+      <c r="D818" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E818" s="2">
+        <v>128</v>
+      </c>
+      <c r="F818" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="G818" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="H818" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="I818" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J818" s="2">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="819" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A819" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B819" s="17">
+        <v>0.4375</v>
+      </c>
+      <c r="C819" s="2" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D819" s="2" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E819" s="2">
+        <v>90</v>
+      </c>
+      <c r="F819" s="2">
+        <v>2</v>
+      </c>
+      <c r="G819" s="2">
+        <v>21</v>
+      </c>
+      <c r="H819" s="2">
+        <v>1</v>
+      </c>
+      <c r="I819" s="2">
+        <v>14</v>
+      </c>
+      <c r="J819" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="820" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A820" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B820" s="17">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C820" s="2" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D820" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E820" s="2">
+        <v>290</v>
+      </c>
+      <c r="F820" s="2">
+        <v>11</v>
+      </c>
+      <c r="G820" s="2">
+        <v>18</v>
+      </c>
+      <c r="H820" s="2">
+        <v>18</v>
+      </c>
+      <c r="I820" s="2">
+        <v>0</v>
+      </c>
+      <c r="J820" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="821" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A821" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B821" s="17">
+        <v>0.625</v>
+      </c>
+      <c r="C821" s="2" t="s">
+        <v>1204</v>
+      </c>
+      <c r="D821" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="E821" s="2">
+        <v>335</v>
+      </c>
+      <c r="F821" s="2">
+        <v>21</v>
+      </c>
+      <c r="G821" s="2">
+        <v>33</v>
+      </c>
+      <c r="H821" s="2">
+        <v>13</v>
+      </c>
+      <c r="I821" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="J821" s="2">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="822" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A822" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B822" s="17">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="C822" s="2" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D822" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E822" s="2">
+        <v>77</v>
+      </c>
+      <c r="F822" s="2">
+        <v>2</v>
+      </c>
+      <c r="G822" s="2">
+        <v>11</v>
+      </c>
+      <c r="H822" s="2">
+        <v>2</v>
+      </c>
+      <c r="I822" s="2">
+        <v>7</v>
+      </c>
+      <c r="J822" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="823" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A823" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B823" s="17">
+        <v>0.75</v>
+      </c>
+      <c r="C823" s="2" t="s">
+        <v>1206</v>
+      </c>
+      <c r="D823" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E823" s="2">
+        <v>380</v>
+      </c>
+      <c r="F823" s="2">
+        <v>25</v>
+      </c>
+      <c r="G823" s="2">
+        <v>46</v>
+      </c>
+      <c r="H823" s="2">
+        <v>10</v>
+      </c>
+      <c r="I823" s="2">
+        <v>2</v>
+      </c>
+      <c r="J823" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="824" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A824" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B824" s="17">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="C824" s="2" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D824" s="2" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E824" s="2">
+        <v>175</v>
+      </c>
+      <c r="F824" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G824" s="2">
+        <v>20</v>
+      </c>
+      <c r="H824" s="2">
+        <v>2</v>
+      </c>
+      <c r="I824" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="J824" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="825" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A825" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B825" s="17">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="C825" s="2" t="s">
+        <v>1209</v>
+      </c>
+      <c r="D825" s="2" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E825" s="2">
+        <v>156</v>
+      </c>
+      <c r="F825" s="2">
+        <v>12.6</v>
+      </c>
+      <c r="G825" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="H825" s="2">
+        <v>10.6</v>
+      </c>
+      <c r="I825" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="J825" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="826" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A826" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B826" s="17">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="C826" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="D826" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E826" s="2">
+        <v>77</v>
+      </c>
+      <c r="F826" s="2">
+        <v>2</v>
+      </c>
+      <c r="G826" s="2">
+        <v>11</v>
+      </c>
+      <c r="H826" s="2">
+        <v>2</v>
+      </c>
+      <c r="I826" s="2">
+        <v>7</v>
+      </c>
+      <c r="J826" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="827" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A827" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B827" s="17">
+        <v>0.3125</v>
+      </c>
+      <c r="C827" s="2" t="s">
+        <v>1211</v>
+      </c>
+      <c r="D827" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E827" s="2">
+        <v>128</v>
+      </c>
+      <c r="F827" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="G827" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="H827" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="I827" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J827" s="2">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="828" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A828" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B828" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C828" s="2" t="s">
+        <v>1212</v>
+      </c>
+      <c r="D828" s="2" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E828" s="2">
+        <v>90</v>
+      </c>
+      <c r="F828" s="2">
+        <v>2</v>
+      </c>
+      <c r="G828" s="2">
+        <v>21</v>
+      </c>
+      <c r="H828" s="2">
+        <v>1</v>
+      </c>
+      <c r="I828" s="2">
+        <v>14</v>
+      </c>
+      <c r="J828" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="829" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A829" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B829" s="17">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="C829" s="2" t="s">
+        <v>1213</v>
+      </c>
+      <c r="D829" s="2" t="s">
+        <v>1214</v>
+      </c>
+      <c r="E829" s="2">
+        <v>175</v>
+      </c>
+      <c r="F829" s="2">
+        <v>4</v>
+      </c>
+      <c r="G829" s="2">
+        <v>28</v>
+      </c>
+      <c r="H829" s="2">
+        <v>6</v>
+      </c>
+      <c r="I829" s="2">
+        <v>12</v>
+      </c>
+      <c r="J829" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="830" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A830" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B830" s="17">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C830" s="2" t="s">
+        <v>1215</v>
+      </c>
+      <c r="D830" s="2" t="s">
+        <v>1216</v>
+      </c>
+      <c r="E830" s="2">
+        <v>90</v>
+      </c>
+      <c r="F830" s="2">
+        <v>3.3</v>
+      </c>
+      <c r="G830" s="2">
+        <v>10</v>
+      </c>
+      <c r="H830" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="I830" s="2">
+        <v>9</v>
+      </c>
+      <c r="J830" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="831" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A831" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B831" s="17">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="C831" s="2" t="s">
+        <v>1217</v>
+      </c>
+      <c r="D831" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E831" s="2">
+        <v>290</v>
+      </c>
+      <c r="F831" s="2">
+        <v>11</v>
+      </c>
+      <c r="G831" s="2">
+        <v>18</v>
+      </c>
+      <c r="H831" s="2">
+        <v>18</v>
+      </c>
+      <c r="I831" s="2">
+        <v>0</v>
+      </c>
+      <c r="J831" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="832" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A832" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B832" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="C832" s="2" t="s">
+        <v>1218</v>
+      </c>
+      <c r="D832" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E832" s="2">
+        <v>155</v>
+      </c>
+      <c r="F832" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="G832" s="2">
+        <v>15</v>
+      </c>
+      <c r="H832" s="2">
+        <v>2</v>
+      </c>
+      <c r="I832" s="2">
+        <v>7</v>
+      </c>
+      <c r="J832" s="2">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="833" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A833" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B833" s="17">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C833" s="2" t="s">
+        <v>1219</v>
+      </c>
+      <c r="D833" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="E833" s="2">
+        <v>145</v>
+      </c>
+      <c r="F833" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="G833" s="2">
+        <v>9</v>
+      </c>
+      <c r="H833" s="2">
+        <v>9</v>
+      </c>
+      <c r="I833" s="2">
+        <v>0</v>
+      </c>
+      <c r="J833" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="834" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A834" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B834" s="17">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C834" s="2" t="s">
+        <v>1220</v>
+      </c>
+      <c r="D834" s="2" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E834" s="2">
+        <v>243</v>
+      </c>
+      <c r="F834" s="2">
+        <v>12</v>
+      </c>
+      <c r="G834" s="2">
+        <v>19</v>
+      </c>
+      <c r="H834" s="2">
+        <v>13</v>
+      </c>
+      <c r="I834" s="2">
+        <v>5</v>
+      </c>
+      <c r="J834" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="835" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A835" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B835" s="17">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="C835" s="2" t="s">
+        <v>1221</v>
+      </c>
+      <c r="D835" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="E835" s="2">
+        <v>335</v>
+      </c>
+      <c r="F835" s="2">
+        <v>21</v>
+      </c>
+      <c r="G835" s="2">
+        <v>33</v>
+      </c>
+      <c r="H835" s="2">
+        <v>13</v>
+      </c>
+      <c r="I835" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="J835" s="2">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="836" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A836" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B836" s="17">
+        <v>0.75</v>
+      </c>
+      <c r="C836" s="2" t="s">
+        <v>1222</v>
+      </c>
+      <c r="D836" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="E836" s="2">
+        <v>270</v>
+      </c>
+      <c r="F836" s="2">
+        <v>6</v>
+      </c>
+      <c r="G836" s="2">
+        <v>35</v>
+      </c>
+      <c r="H836" s="2">
+        <v>12</v>
+      </c>
+      <c r="I836" s="2">
+        <v>1</v>
+      </c>
+      <c r="J836" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="837" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A837" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B837" s="17">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C837" s="2" t="s">
+        <v>1223</v>
+      </c>
+      <c r="D837" s="2" t="s">
+        <v>1224</v>
+      </c>
+      <c r="E837" s="2">
+        <v>158</v>
+      </c>
+      <c r="F837" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="G837" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="H837" s="2">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="I837" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="J837" s="2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="838" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A838" s="16">
+        <v>46038</v>
+      </c>
+      <c r="B838" s="17">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C838" s="2" t="s">
+        <v>1225</v>
+      </c>
+      <c r="D838" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E838" s="2">
+        <v>128</v>
+      </c>
+      <c r="F838" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="G838" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="H838" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="I838" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J838" s="2">
+        <v>2.7</v>
       </c>
     </row>
   </sheetData>
@@ -29876,12 +31072,13 @@
     <cfRule type="duplicateValues" dxfId="0" priority="8"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F24E0C0-BC77-4AA4-801C-82B038A8B8E4}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -30516,16 +31713,16 @@
       <c r="A32" s="16">
         <v>46031</v>
       </c>
-      <c r="B32" s="31">
+      <c r="B32" s="2">
         <v>97.7</v>
       </c>
-      <c r="C32" s="31">
+      <c r="C32" s="2">
         <v>35.9</v>
       </c>
-      <c r="D32" s="31">
+      <c r="D32" s="2">
         <v>30.7</v>
       </c>
-      <c r="E32" s="31">
+      <c r="E32" s="2">
         <v>49.1</v>
       </c>
       <c r="F32" s="2"/>
@@ -30534,16 +31731,16 @@
       <c r="A33" s="16">
         <v>46033</v>
       </c>
-      <c r="B33" s="31">
+      <c r="B33" s="2">
         <v>97.3</v>
       </c>
-      <c r="C33" s="31">
+      <c r="C33" s="2">
         <v>36.4</v>
       </c>
-      <c r="D33" s="31">
+      <c r="D33" s="2">
         <v>29.5</v>
       </c>
-      <c r="E33" s="31">
+      <c r="E33" s="2">
         <v>49.7</v>
       </c>
       <c r="F33" s="2"/>
@@ -30566,6 +31763,86 @@
       </c>
       <c r="F34" s="2" t="s">
         <v>1184</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="16">
+        <v>46025</v>
+      </c>
+      <c r="B35" s="2">
+        <v>97.4</v>
+      </c>
+      <c r="C35" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="D35" s="2">
+        <v>30.5</v>
+      </c>
+      <c r="E35" s="2">
+        <v>49.1</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="16">
+        <v>46031</v>
+      </c>
+      <c r="B36" s="2">
+        <v>97.7</v>
+      </c>
+      <c r="C36" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="D36" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E36" s="2">
+        <v>49.1</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="16">
+        <v>46035</v>
+      </c>
+      <c r="B37" s="2">
+        <v>97.1</v>
+      </c>
+      <c r="C37" s="2">
+        <v>37.1</v>
+      </c>
+      <c r="D37" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E37" s="2">
+        <v>50.4</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="16">
+        <v>46039</v>
+      </c>
+      <c r="B38" s="2">
+        <v>97.5</v>
+      </c>
+      <c r="C38" s="2">
+        <v>37.299999999999997</v>
+      </c>
+      <c r="D38" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E38" s="2">
+        <v>50.6</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>1227</v>
       </c>
     </row>
   </sheetData>
@@ -30576,7 +31853,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06D2F321-D2D4-48D2-B6F9-E306604CF730}">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -31745,6 +33022,94 @@
       <c r="G49" s="2"/>
       <c r="H49" s="2" t="s">
         <v>1183</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" s="16">
+        <v>46036</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D50" s="2">
+        <v>54</v>
+      </c>
+      <c r="E50" s="2">
+        <v>523</v>
+      </c>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2" t="s">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D51" s="2">
+        <v>42</v>
+      </c>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2">
+        <v>2720</v>
+      </c>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2" t="s">
+        <v>1229</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52" s="16">
+        <v>46037</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="D52" s="2">
+        <v>58</v>
+      </c>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2">
+        <v>13520</v>
+      </c>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2" t="s">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53" s="16">
+        <v>46039</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D53" s="2">
+        <v>50</v>
+      </c>
+      <c r="E53" s="2">
+        <v>490</v>
+      </c>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2" t="s">
+        <v>1231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>